<commit_message>
FN Korrektur / Fehler in der Prozentuierung
</commit_message>
<xml_diff>
--- a/assets/excel/2026_6-3-1.xlsx
+++ b/assets/excel/2026_6-3-1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr codeName="DieseArbeitsmappe" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\Hannover\Dez15_Uebergreifende_Analysen\Projekte\Integrationsmonitoring\Schlesier\MT_Site\assets\excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\BiesterChristophLSN\Desktop\MZ\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32CF31D2-5072-4EDF-B983-268934BDB332}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{EED34A05-2686-4678-9FA0-CD53D7D61E19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{26AA0D46-F1BF-4408-A6F5-D4E9B3798D9B}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15270" xr2:uid="{26AA0D46-F1BF-4408-A6F5-D4E9B3798D9B}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="2" r:id="rId1"/>
@@ -104,15 +104,6 @@
     <t>Prozent</t>
   </si>
   <si>
-    <t>1) Seit dem Jahr 2018 wird im Mikrozensus der Migrationshintergrund im weiteren Sinne jährlich berichtet. Die in der Tabelle ab dem Jahr 2018 abgebildeten Daten zum Migrationshintergrund entsprechen dem Migrationshintergrund im weiteren Sinne, bis 2017 wird der Migrationshintergrund im engeren Sinne abgebildet. Die Vergleichbarkeit ist dadurch eingeschränkt.</t>
-  </si>
-  <si>
-    <t>2) Einschl. Grundsicherung im Alter und bei Erwerbsminderung und andere Hilfen in besonderen Lebenslagen.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3) Die Ergebnisse des Mikrozensus 2020 sind unter anderem aufgrund methodischer Effekte im Rahmen einer Neugestaltung der Erhebung sowie insbesondere aufgrund der Folgen der Corona-Pandemie in Ihrer Datenqualität eingeschränkt. Auf die Verwendung dieser Ergebnisse wird daher verzichtet. Weitere Informationen zur methodischen Neugestaltung des Mikrozensus ab 2020 und zu den Auswirkungen der Neugestaltung und der Corona-Krise auf die Ergebnisse des Jahres 2020 finden Sie auf der Informationsseite des Statistischen Bundesamtes: </t>
-  </si>
-  <si>
     <t>https://www.destatis.de/DE/Themen/Gesellschaft-Umwelt/Bevoelkerung/Haushalte-Familien/Methoden/mikrozensus-2020.html</t>
   </si>
   <si>
@@ -131,19 +122,27 @@
     <t>Migration und Teilhabe in Niedersachsen - Integrationsmonitoring 2026</t>
   </si>
   <si>
-    <t>© Landesamt für Statistik Niedersachsen, Hannover 2026,                                                                          </t>
+    <t>1)  Ab der Veröffentlichung der Endergebnisse 2023 und der Erstergebnisse 2024 werden für die Hochrechnung des Mikrozensus Daten der Bevölkerungsfortschreibung herangezogen, die auf den Eckwerten des Zensus 2022 basieren. Die Hochrechnung für die Jahre vor 2011 sowie für bislang veröffentlichte Ergebnisse des Mikrozensus 2011-2013 basiert auf den fortgeschriebenen Ergebnissen der Volkszählung 1987. In 2016 erfolgte die Umstellung auf eine neue Mikrozensus-Stichprobe (auf Basis des Zensus 2011). Ab 2017 wird nur noch die Bevölkerung in Privathaushalten (ohne Gemeinschaftsunterkünfte) ausgewiesen. Dadurch ergibt sich jeweils eine eingeschränkte Vergleichbarkeit mit den Vorjahren.</t>
+  </si>
+  <si>
+    <t>2) Seit dem Jahr 2018 wird im Mikrozensus der Migrationshintergrund im weiteren Sinne jährlich berichtet. Die in der Tabelle ab dem Jahr 2018 abgebildeten Daten zum Migrationshintergrund entsprechen dem Migrationshintergrund im weiteren Sinne, bis 2017 wird der Migrationshintergrund im engeren Sinne abgebildet. Die Vergleichbarkeit ist dadurch eingeschränkt.</t>
+  </si>
+  <si>
+    <t>3) Die Ergebnisse des Mikrozensus 2020 sind unter anderem aufgrund methodischer Effekte im Rahmen einer Neugestaltung der Erhebung sowie insbesondere aufgrund der Folgen der Corona-Pandemie in Ihrer Datenqualität eingeschränkt. Auf die Verwendung dieser Ergebnisse wird daher verzichtet. Weitere Informationen zur methodischen Neugestaltung des Mikrozensus ab 2020 und zu den Auswirkungen der Neugestaltung und der Corona-Krise auf die Ergebnisse des Jahres 2020 finden Sie auf der Informationsseite des Statistischen Bundesamtes:</t>
+  </si>
+  <si>
+    <t>© Landesamt für Statistik Niedersachsen, Hannover 2026,</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="3">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="#\ ##0.0"/>
     <numFmt numFmtId="165" formatCode="#,##0.0"/>
-    <numFmt numFmtId="166" formatCode="0.0"/>
   </numFmts>
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -193,10 +192,6 @@
       <sz val="6"/>
       <color theme="10"/>
       <name val="NDSFrutiger 45 Light"/>
-    </font>
-    <font>
-      <sz val="6"/>
-      <name val="NDSFrutiger 55 Roman"/>
     </font>
   </fonts>
   <fills count="2">
@@ -297,7 +292,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="2"/>
@@ -320,26 +315,12 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="3" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="3"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="3" applyFont="1"/>
-    <xf numFmtId="166" fontId="9" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -349,12 +330,6 @@
     </xf>
     <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -371,6 +346,20 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Link" xfId="1" builtinId="8"/>
@@ -392,9 +381,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 – 2022-Design">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 – 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -432,7 +421,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 – 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -538,7 +527,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 – 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -680,7 +669,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -688,6 +677,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{75ADC1A0-2E9E-4486-AEF7-FD006F785543}">
+  <sheetPr codeName="Tabelle1"/>
   <dimension ref="A1:M85"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -697,7 +687,7 @@
   <sheetData>
     <row r="1" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B1" s="1" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="C1" s="2"/>
       <c r="D1" s="2"/>
@@ -742,25 +732,25 @@
       <c r="I4" s="4"/>
     </row>
     <row r="6" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="23" t="s">
+      <c r="B6" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="C6" s="23" t="s">
+      <c r="C6" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="D6" s="26" t="s">
+      <c r="D6" s="18" t="s">
         <v>4</v>
       </c>
-      <c r="E6" s="27"/>
-      <c r="F6" s="27"/>
-      <c r="G6" s="27"/>
-      <c r="H6" s="27"/>
-      <c r="I6" s="27"/>
-      <c r="J6" s="27"/>
+      <c r="E6" s="19"/>
+      <c r="F6" s="19"/>
+      <c r="G6" s="19"/>
+      <c r="H6" s="19"/>
+      <c r="I6" s="19"/>
+      <c r="J6" s="19"/>
     </row>
     <row r="7" spans="2:10" ht="41.25" x14ac:dyDescent="0.25">
-      <c r="B7" s="24"/>
-      <c r="C7" s="24"/>
+      <c r="B7" s="16"/>
+      <c r="C7" s="16"/>
       <c r="D7" s="5" t="s">
         <v>5</v>
       </c>
@@ -784,908 +774,908 @@
       </c>
     </row>
     <row r="8" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B8" s="25"/>
-      <c r="C8" s="25"/>
-      <c r="D8" s="26" t="s">
+      <c r="B8" s="17"/>
+      <c r="C8" s="17"/>
+      <c r="D8" s="18" t="s">
         <v>12</v>
       </c>
-      <c r="E8" s="27"/>
-      <c r="F8" s="27"/>
-      <c r="G8" s="27"/>
-      <c r="H8" s="27"/>
-      <c r="I8" s="27"/>
-      <c r="J8" s="27"/>
+      <c r="E8" s="19"/>
+      <c r="F8" s="19"/>
+      <c r="G8" s="19"/>
+      <c r="H8" s="19"/>
+      <c r="I8" s="19"/>
+      <c r="J8" s="19"/>
     </row>
     <row r="9" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="18" t="s">
-        <v>13</v>
-      </c>
-      <c r="C9" s="18">
+      <c r="B9" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="C9" s="12">
         <v>2025</v>
       </c>
-      <c r="D9" s="19">
+      <c r="D9" s="13">
         <v>5784.797157</v>
       </c>
-      <c r="E9" s="19">
+      <c r="E9" s="13">
         <v>2646.5485319999998</v>
       </c>
-      <c r="F9" s="19">
+      <c r="F9" s="13">
         <v>168.91743099999999</v>
       </c>
-      <c r="G9" s="19">
+      <c r="G9" s="13">
         <v>1573.325758</v>
       </c>
-      <c r="H9" s="19">
+      <c r="H9" s="13">
         <v>1142.722673</v>
       </c>
-      <c r="I9" s="19">
+      <c r="I9" s="13">
         <v>55.312877999999998</v>
       </c>
-      <c r="J9" s="19">
+      <c r="J9" s="13">
         <v>197.969885</v>
       </c>
     </row>
     <row r="10" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="C10" s="18">
+      <c r="B10" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C10" s="12">
         <v>2025</v>
       </c>
-      <c r="D10" s="19">
+      <c r="D10" s="13">
         <v>2127.741853</v>
       </c>
-      <c r="E10" s="19">
+      <c r="E10" s="13">
         <v>895.07401300000004</v>
       </c>
-      <c r="F10" s="19">
+      <c r="F10" s="13">
         <v>247.47972300000001</v>
       </c>
-      <c r="G10" s="19">
+      <c r="G10" s="13">
         <v>204.98495</v>
       </c>
-      <c r="H10" s="19">
+      <c r="H10" s="13">
         <v>611.61364300000002</v>
       </c>
-      <c r="I10" s="19">
+      <c r="I10" s="13">
         <v>55.849573999999997</v>
       </c>
-      <c r="J10" s="19">
+      <c r="J10" s="13">
         <v>112.73994999999999</v>
       </c>
     </row>
     <row r="11" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="18" t="s">
-        <v>13</v>
-      </c>
-      <c r="C11" s="18">
+      <c r="B11" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="C11" s="12">
         <v>2024</v>
       </c>
-      <c r="D11" s="19">
+      <c r="D11" s="13">
         <v>5812.2569389999999</v>
       </c>
-      <c r="E11" s="19">
+      <c r="E11" s="13">
         <v>2667.337149</v>
       </c>
-      <c r="F11" s="19">
+      <c r="F11" s="13">
         <v>155.398888</v>
       </c>
-      <c r="G11" s="19">
+      <c r="G11" s="13">
         <v>1568.245365</v>
       </c>
-      <c r="H11" s="19">
+      <c r="H11" s="13">
         <v>1168.5717070000001</v>
       </c>
-      <c r="I11" s="19">
+      <c r="I11" s="13">
         <v>58.119768999999998</v>
       </c>
-      <c r="J11" s="19">
+      <c r="J11" s="13">
         <v>194.58406099999996</v>
       </c>
     </row>
     <row r="12" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B12" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="C12" s="18">
+      <c r="B12" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C12" s="12">
         <v>2024</v>
       </c>
-      <c r="D12" s="19">
+      <c r="D12" s="13">
         <v>2108.566898</v>
       </c>
-      <c r="E12" s="19">
+      <c r="E12" s="13">
         <v>875.358428</v>
       </c>
-      <c r="F12" s="19">
+      <c r="F12" s="13">
         <v>247.13717600000001</v>
       </c>
-      <c r="G12" s="19">
+      <c r="G12" s="13">
         <v>210.193262</v>
       </c>
-      <c r="H12" s="19">
+      <c r="H12" s="13">
         <v>602.84329100000002</v>
       </c>
-      <c r="I12" s="19">
+      <c r="I12" s="13">
         <v>61.026826999999997</v>
       </c>
-      <c r="J12" s="19">
+      <c r="J12" s="13">
         <v>112.007914</v>
       </c>
     </row>
     <row r="13" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B13" s="18" t="s">
-        <v>13</v>
-      </c>
-      <c r="C13" s="18">
+      <c r="B13" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="C13" s="12">
         <v>2023</v>
       </c>
-      <c r="D13" s="19">
+      <c r="D13" s="13">
         <v>5927.2500280000013</v>
       </c>
-      <c r="E13" s="19">
+      <c r="E13" s="13">
         <v>2737.2947330000002</v>
       </c>
-      <c r="F13" s="19">
+      <c r="F13" s="13">
         <v>159.35100299999999</v>
       </c>
-      <c r="G13" s="19">
+      <c r="G13" s="13">
         <v>1567.4829970000001</v>
       </c>
-      <c r="H13" s="19">
+      <c r="H13" s="13">
         <v>1212.2092700000001</v>
       </c>
-      <c r="I13" s="19">
+      <c r="I13" s="13">
         <v>57.388255999999998</v>
       </c>
-      <c r="J13" s="19">
+      <c r="J13" s="13">
         <v>193.52376899999999</v>
       </c>
     </row>
     <row r="14" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="C14" s="18">
+      <c r="B14" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C14" s="12">
         <v>2023</v>
       </c>
-      <c r="D14" s="19">
+      <c r="D14" s="13">
         <v>1977.1603669999997</v>
       </c>
-      <c r="E14" s="19">
+      <c r="E14" s="13">
         <v>808.59620299999995</v>
       </c>
-      <c r="F14" s="19">
+      <c r="F14" s="13">
         <v>248.42204699999999</v>
       </c>
-      <c r="G14" s="19">
+      <c r="G14" s="13">
         <v>190.69550699999999</v>
       </c>
-      <c r="H14" s="19">
+      <c r="H14" s="13">
         <v>585.40226900000005</v>
       </c>
-      <c r="I14" s="19">
+      <c r="I14" s="13">
         <v>47.727291000000001</v>
       </c>
-      <c r="J14" s="19">
+      <c r="J14" s="13">
         <v>96.317050000000009</v>
       </c>
     </row>
     <row r="15" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="18" t="s">
-        <v>13</v>
-      </c>
-      <c r="C15" s="18">
+      <c r="B15" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="C15" s="12">
         <v>2022</v>
       </c>
-      <c r="D15" s="19">
+      <c r="D15" s="13">
         <v>5949.9528930000006</v>
       </c>
-      <c r="E15" s="19">
+      <c r="E15" s="13">
         <v>2712.6327620000002</v>
       </c>
-      <c r="F15" s="19">
+      <c r="F15" s="13">
         <v>156.03676999999999</v>
       </c>
-      <c r="G15" s="19">
+      <c r="G15" s="13">
         <v>1577.6182859999999</v>
       </c>
-      <c r="H15" s="19">
+      <c r="H15" s="13">
         <v>1240.333085</v>
       </c>
-      <c r="I15" s="19">
+      <c r="I15" s="13">
         <v>48.281765999999998</v>
       </c>
-      <c r="J15" s="19">
+      <c r="J15" s="13">
         <v>215.05022400000001</v>
       </c>
     </row>
     <row r="16" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B16" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="C16" s="18">
+      <c r="B16" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C16" s="12">
         <v>2022</v>
       </c>
-      <c r="D16" s="19">
+      <c r="D16" s="13">
         <v>1901.0437259999999</v>
       </c>
-      <c r="E16" s="19">
+      <c r="E16" s="13">
         <v>791.63186599999995</v>
       </c>
-      <c r="F16" s="19">
+      <c r="F16" s="13">
         <v>194.831391</v>
       </c>
-      <c r="G16" s="19">
+      <c r="G16" s="13">
         <v>185.826784</v>
       </c>
-      <c r="H16" s="19">
+      <c r="H16" s="13">
         <v>603.31300699999997</v>
       </c>
-      <c r="I16" s="19">
+      <c r="I16" s="13">
         <v>42.077596999999997</v>
       </c>
-      <c r="J16" s="19">
+      <c r="J16" s="13">
         <v>83.363081000000008</v>
       </c>
     </row>
     <row r="17" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="18" t="s">
-        <v>13</v>
-      </c>
-      <c r="C17" s="18">
+      <c r="B17" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="C17" s="12">
         <v>2021</v>
       </c>
-      <c r="D17" s="19">
+      <c r="D17" s="13">
         <v>5944.9624909999984</v>
       </c>
-      <c r="E17" s="19">
+      <c r="E17" s="13">
         <v>2709.629359</v>
       </c>
-      <c r="F17" s="19">
+      <c r="F17" s="13">
         <v>157.81235699999999</v>
       </c>
-      <c r="G17" s="19">
+      <c r="G17" s="13">
         <v>1558.9248250000001</v>
       </c>
-      <c r="H17" s="19">
+      <c r="H17" s="13">
         <v>1260.374069</v>
       </c>
-      <c r="I17" s="19">
+      <c r="I17" s="13">
         <v>49.197209000000001</v>
       </c>
-      <c r="J17" s="19">
+      <c r="J17" s="13">
         <v>209.02467199999998</v>
       </c>
     </row>
     <row r="18" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="C18" s="18">
+      <c r="B18" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C18" s="12">
         <v>2021</v>
       </c>
-      <c r="D18" s="19">
+      <c r="D18" s="13">
         <v>1806.6768549999999</v>
       </c>
-      <c r="E18" s="19">
+      <c r="E18" s="13">
         <v>739.63828000000001</v>
       </c>
-      <c r="F18" s="19">
+      <c r="F18" s="13">
         <v>164.25168600000001</v>
       </c>
-      <c r="G18" s="19">
+      <c r="G18" s="13">
         <v>190.715597</v>
       </c>
-      <c r="H18" s="19">
+      <c r="H18" s="13">
         <v>596.98005899999998</v>
       </c>
-      <c r="I18" s="19">
+      <c r="I18" s="13">
         <v>33.904470000000003</v>
       </c>
-      <c r="J18" s="19">
+      <c r="J18" s="13">
         <v>81.186762999999999</v>
       </c>
     </row>
     <row r="19" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B19" s="18" t="s">
-        <v>13</v>
-      </c>
-      <c r="C19" s="18">
+      <c r="B19" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="C19" s="12">
         <v>2020</v>
       </c>
-      <c r="D19" s="19">
+      <c r="D19" s="13">
         <v>6097</v>
       </c>
-      <c r="E19" s="19">
+      <c r="E19" s="13">
         <v>2877</v>
       </c>
-      <c r="F19" s="19">
+      <c r="F19" s="13">
         <v>131</v>
       </c>
-      <c r="G19" s="19">
+      <c r="G19" s="13">
         <v>1636</v>
       </c>
-      <c r="H19" s="19">
+      <c r="H19" s="13">
         <v>1205</v>
       </c>
-      <c r="I19" s="19">
+      <c r="I19" s="13">
         <v>39</v>
       </c>
-      <c r="J19" s="19">
+      <c r="J19" s="13">
         <v>209</v>
       </c>
     </row>
     <row r="20" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="C20" s="18">
+      <c r="B20" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C20" s="12">
         <v>2020</v>
       </c>
-      <c r="D20" s="19">
+      <c r="D20" s="13">
         <v>1798</v>
       </c>
-      <c r="E20" s="19">
+      <c r="E20" s="13">
         <v>760</v>
       </c>
-      <c r="F20" s="19">
+      <c r="F20" s="13">
         <v>169</v>
       </c>
-      <c r="G20" s="19">
+      <c r="G20" s="13">
         <v>176</v>
       </c>
-      <c r="H20" s="19">
+      <c r="H20" s="13">
         <v>547</v>
       </c>
-      <c r="I20" s="19">
+      <c r="I20" s="13">
         <v>41</v>
       </c>
-      <c r="J20" s="19">
+      <c r="J20" s="13">
         <v>105</v>
       </c>
     </row>
     <row r="21" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="18" t="s">
-        <v>13</v>
-      </c>
-      <c r="C21" s="18">
+      <c r="B21" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="C21" s="12">
         <v>2019</v>
       </c>
-      <c r="D21" s="19">
+      <c r="D21" s="13">
         <v>6103.5</v>
       </c>
-      <c r="E21" s="19">
+      <c r="E21" s="13">
         <v>2876.7</v>
       </c>
-      <c r="F21" s="19">
+      <c r="F21" s="13">
         <v>150.4</v>
       </c>
-      <c r="G21" s="19">
+      <c r="G21" s="13">
         <v>1534.6</v>
       </c>
-      <c r="H21" s="19">
+      <c r="H21" s="13">
         <v>1362.4</v>
       </c>
-      <c r="I21" s="19">
+      <c r="I21" s="13">
         <v>39</v>
       </c>
-      <c r="J21" s="19">
+      <c r="J21" s="13">
         <v>140.4</v>
       </c>
     </row>
     <row r="22" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B22" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="C22" s="18">
+      <c r="B22" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C22" s="12">
         <v>2019</v>
       </c>
-      <c r="D22" s="19">
+      <c r="D22" s="13">
         <v>1786.4</v>
       </c>
-      <c r="E22" s="19">
+      <c r="E22" s="13">
         <v>727.7</v>
       </c>
-      <c r="F22" s="19">
+      <c r="F22" s="13">
         <v>135.5</v>
       </c>
-      <c r="G22" s="19">
+      <c r="G22" s="13">
         <v>167.3</v>
       </c>
-      <c r="H22" s="19">
+      <c r="H22" s="13">
         <v>625.79999999999995</v>
       </c>
-      <c r="I22" s="19">
+      <c r="I22" s="13">
         <v>40.200000000000003</v>
       </c>
-      <c r="J22" s="19">
+      <c r="J22" s="13">
         <v>89.9</v>
       </c>
     </row>
     <row r="23" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="18" t="s">
-        <v>13</v>
-      </c>
-      <c r="C23" s="18">
+      <c r="B23" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="C23" s="12">
         <v>2018</v>
       </c>
-      <c r="D23" s="19">
+      <c r="D23" s="13">
         <v>6106.2</v>
       </c>
-      <c r="E23" s="19">
+      <c r="E23" s="13">
         <v>2833.6</v>
       </c>
-      <c r="F23" s="19">
+      <c r="F23" s="13">
         <v>155.69999999999999</v>
       </c>
-      <c r="G23" s="19">
+      <c r="G23" s="13">
         <v>1538.7</v>
       </c>
-      <c r="H23" s="19">
+      <c r="H23" s="13">
         <v>1405.5</v>
       </c>
-      <c r="I23" s="19">
+      <c r="I23" s="13">
         <v>31.8</v>
       </c>
-      <c r="J23" s="19">
+      <c r="J23" s="13">
         <v>140.9</v>
       </c>
     </row>
     <row r="24" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B24" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="C24" s="18">
+      <c r="B24" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C24" s="12">
         <v>2018</v>
       </c>
-      <c r="D24" s="19">
+      <c r="D24" s="13">
         <v>1761.3000000000002</v>
       </c>
-      <c r="E24" s="19">
+      <c r="E24" s="13">
         <v>713.1</v>
       </c>
-      <c r="F24" s="19">
+      <c r="F24" s="13">
         <v>134.4</v>
       </c>
-      <c r="G24" s="19">
+      <c r="G24" s="13">
         <v>159.19999999999999</v>
       </c>
-      <c r="H24" s="19">
+      <c r="H24" s="13">
         <v>624.20000000000005</v>
       </c>
-      <c r="I24" s="19">
+      <c r="I24" s="13">
         <v>40.9</v>
       </c>
-      <c r="J24" s="19">
+      <c r="J24" s="13">
         <v>89.5</v>
       </c>
     </row>
     <row r="25" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="18" t="s">
-        <v>13</v>
-      </c>
-      <c r="C25" s="18">
+      <c r="B25" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="C25" s="12">
         <v>2017</v>
       </c>
-      <c r="D25" s="19">
+      <c r="D25" s="13">
         <v>6227</v>
       </c>
-      <c r="E25" s="19">
+      <c r="E25" s="13">
         <v>2869</v>
       </c>
-      <c r="F25" s="19">
+      <c r="F25" s="13">
         <v>164</v>
       </c>
-      <c r="G25" s="19">
+      <c r="G25" s="13">
         <v>1515</v>
       </c>
-      <c r="H25" s="19">
+      <c r="H25" s="13">
         <v>1451</v>
       </c>
-      <c r="I25" s="19">
+      <c r="I25" s="13">
         <v>43</v>
       </c>
-      <c r="J25" s="19">
+      <c r="J25" s="13">
         <v>185</v>
       </c>
     </row>
     <row r="26" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B26" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="C26" s="18">
+      <c r="B26" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C26" s="12">
         <v>2017</v>
       </c>
-      <c r="D26" s="19">
+      <c r="D26" s="13">
         <v>1701</v>
       </c>
-      <c r="E26" s="19">
+      <c r="E26" s="13">
         <v>642</v>
       </c>
-      <c r="F26" s="19">
+      <c r="F26" s="13">
         <v>123</v>
       </c>
-      <c r="G26" s="19">
+      <c r="G26" s="13">
         <v>160</v>
       </c>
-      <c r="H26" s="19">
+      <c r="H26" s="13">
         <v>612</v>
       </c>
-      <c r="I26" s="19">
+      <c r="I26" s="13">
         <v>46</v>
       </c>
-      <c r="J26" s="19">
+      <c r="J26" s="13">
         <v>118</v>
       </c>
     </row>
     <row r="27" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B27" s="18" t="s">
-        <v>13</v>
-      </c>
-      <c r="C27" s="18">
+      <c r="B27" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="C27" s="12">
         <v>2016</v>
       </c>
-      <c r="D27" s="19">
+      <c r="D27" s="13">
         <v>6399</v>
       </c>
-      <c r="E27" s="19">
+      <c r="E27" s="13">
         <v>2881</v>
       </c>
-      <c r="F27" s="19">
+      <c r="F27" s="13">
         <v>178</v>
       </c>
-      <c r="G27" s="19">
+      <c r="G27" s="13">
         <v>1593</v>
       </c>
-      <c r="H27" s="19">
+      <c r="H27" s="13">
         <v>1547</v>
       </c>
-      <c r="I27" s="19">
+      <c r="I27" s="13">
         <v>62</v>
       </c>
-      <c r="J27" s="19">
+      <c r="J27" s="13">
         <v>138</v>
       </c>
     </row>
     <row r="28" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B28" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="C28" s="18">
+      <c r="B28" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C28" s="12">
         <v>2016</v>
       </c>
-      <c r="D28" s="19">
+      <c r="D28" s="13">
         <v>1594</v>
       </c>
-      <c r="E28" s="19">
+      <c r="E28" s="13">
         <v>594</v>
       </c>
-      <c r="F28" s="19">
+      <c r="F28" s="13">
         <v>108</v>
       </c>
-      <c r="G28" s="19">
+      <c r="G28" s="13">
         <v>152</v>
       </c>
-      <c r="H28" s="19">
+      <c r="H28" s="13">
         <v>585</v>
       </c>
-      <c r="I28" s="19">
+      <c r="I28" s="13">
         <v>55</v>
       </c>
-      <c r="J28" s="19">
+      <c r="J28" s="13">
         <v>100</v>
       </c>
     </row>
     <row r="29" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B29" s="18" t="s">
-        <v>13</v>
-      </c>
-      <c r="C29" s="18">
+      <c r="B29" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="C29" s="12">
         <v>2015</v>
       </c>
-      <c r="D29" s="19">
+      <c r="D29" s="13">
         <v>6457</v>
       </c>
-      <c r="E29" s="19">
+      <c r="E29" s="13">
         <v>2863</v>
       </c>
-      <c r="F29" s="19">
+      <c r="F29" s="13">
         <v>202</v>
       </c>
-      <c r="G29" s="19">
+      <c r="G29" s="13">
         <v>1608</v>
       </c>
-      <c r="H29" s="19">
+      <c r="H29" s="13">
         <v>1591</v>
       </c>
-      <c r="I29" s="19">
+      <c r="I29" s="13">
         <v>54</v>
       </c>
-      <c r="J29" s="19">
+      <c r="J29" s="13">
         <v>139</v>
       </c>
     </row>
     <row r="30" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B30" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="C30" s="18">
+      <c r="B30" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C30" s="12">
         <v>2015</v>
       </c>
-      <c r="D30" s="19">
+      <c r="D30" s="13">
         <v>1408</v>
       </c>
-      <c r="E30" s="19">
+      <c r="E30" s="13">
         <v>532</v>
       </c>
-      <c r="F30" s="19">
+      <c r="F30" s="13">
         <v>112</v>
       </c>
-      <c r="G30" s="19">
+      <c r="G30" s="13">
         <v>143</v>
       </c>
-      <c r="H30" s="19">
+      <c r="H30" s="13">
         <v>540</v>
       </c>
-      <c r="I30" s="19">
+      <c r="I30" s="13">
         <v>40</v>
       </c>
-      <c r="J30" s="19">
+      <c r="J30" s="13">
         <v>41</v>
       </c>
     </row>
     <row r="31" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B31" s="18" t="s">
-        <v>13</v>
-      </c>
-      <c r="C31" s="18">
+      <c r="B31" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="C31" s="12">
         <v>2014</v>
       </c>
-      <c r="D31" s="19">
+      <c r="D31" s="13">
         <v>6429</v>
       </c>
-      <c r="E31" s="19">
+      <c r="E31" s="13">
         <v>2820</v>
       </c>
-      <c r="F31" s="19">
+      <c r="F31" s="13">
         <v>211</v>
       </c>
-      <c r="G31" s="19">
+      <c r="G31" s="13">
         <v>1575</v>
       </c>
-      <c r="H31" s="19">
+      <c r="H31" s="13">
         <v>1657</v>
       </c>
-      <c r="I31" s="19">
+      <c r="I31" s="13">
         <v>62</v>
       </c>
-      <c r="J31" s="19">
+      <c r="J31" s="13">
         <v>104</v>
       </c>
     </row>
     <row r="32" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B32" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="C32" s="18">
+      <c r="B32" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C32" s="12">
         <v>2014</v>
       </c>
-      <c r="D32" s="19">
+      <c r="D32" s="13">
         <v>1362</v>
       </c>
-      <c r="E32" s="19">
+      <c r="E32" s="13">
         <v>520</v>
       </c>
-      <c r="F32" s="19">
+      <c r="F32" s="13">
         <v>99</v>
       </c>
-      <c r="G32" s="19">
+      <c r="G32" s="13">
         <v>140</v>
       </c>
-      <c r="H32" s="19">
+      <c r="H32" s="13">
         <v>547</v>
       </c>
-      <c r="I32" s="19">
+      <c r="I32" s="13">
         <v>30</v>
       </c>
-      <c r="J32" s="19">
+      <c r="J32" s="13">
         <v>26</v>
       </c>
     </row>
     <row r="33" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B33" s="18" t="s">
-        <v>13</v>
-      </c>
-      <c r="C33" s="18">
+      <c r="B33" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="C33" s="12">
         <v>2013</v>
       </c>
-      <c r="D33" s="19">
+      <c r="D33" s="13">
         <v>6373</v>
       </c>
-      <c r="E33" s="19">
+      <c r="E33" s="13">
         <v>2761</v>
       </c>
-      <c r="F33" s="19">
+      <c r="F33" s="13">
         <v>211</v>
       </c>
-      <c r="G33" s="19">
+      <c r="G33" s="13">
         <v>1581</v>
       </c>
-      <c r="H33" s="19">
+      <c r="H33" s="13">
         <v>1683</v>
       </c>
-      <c r="I33" s="19">
+      <c r="I33" s="13">
         <v>45</v>
       </c>
-      <c r="J33" s="19">
+      <c r="J33" s="13">
         <v>92</v>
       </c>
     </row>
     <row r="34" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B34" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="C34" s="18">
+      <c r="B34" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C34" s="12">
         <v>2013</v>
       </c>
-      <c r="D34" s="19">
+      <c r="D34" s="13">
         <v>1409</v>
       </c>
-      <c r="E34" s="19">
+      <c r="E34" s="13">
         <v>550</v>
       </c>
-      <c r="F34" s="19">
+      <c r="F34" s="13">
         <v>110</v>
       </c>
-      <c r="G34" s="19">
+      <c r="G34" s="13">
         <v>137</v>
       </c>
-      <c r="H34" s="19">
+      <c r="H34" s="13">
         <v>557</v>
       </c>
-      <c r="I34" s="19">
+      <c r="I34" s="13">
         <v>25</v>
       </c>
-      <c r="J34" s="19">
+      <c r="J34" s="13">
         <v>30</v>
       </c>
     </row>
     <row r="35" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B35" s="18" t="s">
-        <v>13</v>
-      </c>
-      <c r="C35" s="18">
+      <c r="B35" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="C35" s="12">
         <v>2012</v>
       </c>
-      <c r="D35" s="19">
+      <c r="D35" s="13">
         <v>6490</v>
       </c>
-      <c r="E35" s="19">
+      <c r="E35" s="13">
         <v>2787</v>
       </c>
-      <c r="F35" s="19">
+      <c r="F35" s="13">
         <v>214</v>
       </c>
-      <c r="G35" s="19">
+      <c r="G35" s="13">
         <v>1577</v>
       </c>
-      <c r="H35" s="19">
+      <c r="H35" s="13">
         <v>1727</v>
       </c>
-      <c r="I35" s="19">
+      <c r="I35" s="13">
         <v>49</v>
       </c>
-      <c r="J35" s="19">
+      <c r="J35" s="13">
         <v>136</v>
       </c>
     </row>
     <row r="36" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B36" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="C36" s="18">
+      <c r="B36" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C36" s="12">
         <v>2012</v>
       </c>
-      <c r="D36" s="19">
+      <c r="D36" s="13">
         <v>1311</v>
       </c>
-      <c r="E36" s="19">
+      <c r="E36" s="13">
         <v>488</v>
       </c>
-      <c r="F36" s="19">
+      <c r="F36" s="13">
         <v>103</v>
       </c>
-      <c r="G36" s="19">
+      <c r="G36" s="13">
         <v>131</v>
       </c>
-      <c r="H36" s="19">
+      <c r="H36" s="13">
         <v>528</v>
       </c>
-      <c r="I36" s="19">
+      <c r="I36" s="13">
         <v>25</v>
       </c>
-      <c r="J36" s="19">
+      <c r="J36" s="13">
         <v>36</v>
       </c>
     </row>
     <row r="37" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B37" s="18" t="s">
-        <v>13</v>
-      </c>
-      <c r="C37" s="18">
+      <c r="B37" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="C37" s="12">
         <v>2011</v>
       </c>
-      <c r="D37" s="19">
+      <c r="D37" s="13">
         <v>6517</v>
       </c>
-      <c r="E37" s="19">
+      <c r="E37" s="13">
         <v>2794</v>
       </c>
-      <c r="F37" s="19">
+      <c r="F37" s="13">
         <v>232</v>
       </c>
-      <c r="G37" s="19">
+      <c r="G37" s="13">
         <v>1593</v>
       </c>
-      <c r="H37" s="19">
+      <c r="H37" s="13">
         <v>1714</v>
       </c>
-      <c r="I37" s="19">
+      <c r="I37" s="13">
         <v>51</v>
       </c>
-      <c r="J37" s="19">
+      <c r="J37" s="13">
         <v>133</v>
       </c>
     </row>
     <row r="38" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B38" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="C38" s="18">
+      <c r="B38" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C38" s="12">
         <v>2011</v>
       </c>
-      <c r="D38" s="19">
+      <c r="D38" s="13">
         <v>1273</v>
       </c>
-      <c r="E38" s="19">
+      <c r="E38" s="13">
         <v>473</v>
       </c>
-      <c r="F38" s="19">
+      <c r="F38" s="13">
         <v>112</v>
       </c>
-      <c r="G38" s="19">
+      <c r="G38" s="13">
         <v>126</v>
       </c>
-      <c r="H38" s="19">
+      <c r="H38" s="13">
         <v>504</v>
       </c>
-      <c r="I38" s="19">
+      <c r="I38" s="13">
         <v>28</v>
       </c>
-      <c r="J38" s="19">
+      <c r="J38" s="13">
         <v>30</v>
       </c>
     </row>
     <row r="41" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B41" s="23" t="s">
+      <c r="B41" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="C41" s="23" t="s">
+      <c r="C41" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="D41" s="26" t="s">
+      <c r="D41" s="18" t="s">
         <v>4</v>
       </c>
-      <c r="E41" s="27"/>
-      <c r="F41" s="27"/>
-      <c r="G41" s="27"/>
-      <c r="H41" s="27"/>
-      <c r="I41" s="27"/>
-      <c r="J41" s="27"/>
+      <c r="E41" s="19"/>
+      <c r="F41" s="19"/>
+      <c r="G41" s="19"/>
+      <c r="H41" s="19"/>
+      <c r="I41" s="19"/>
+      <c r="J41" s="19"/>
     </row>
     <row r="42" spans="2:10" ht="41.25" x14ac:dyDescent="0.25">
-      <c r="B42" s="24"/>
-      <c r="C42" s="24"/>
+      <c r="B42" s="16"/>
+      <c r="C42" s="16"/>
       <c r="D42" s="5" t="s">
         <v>5</v>
       </c>
@@ -1709,1066 +1699,1097 @@
       </c>
     </row>
     <row r="43" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B43" s="25"/>
-      <c r="C43" s="25"/>
-      <c r="D43" s="26" t="s">
+      <c r="B43" s="17"/>
+      <c r="C43" s="17"/>
+      <c r="D43" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="E43" s="27"/>
-      <c r="F43" s="27"/>
-      <c r="G43" s="27"/>
-      <c r="H43" s="27"/>
-      <c r="I43" s="27"/>
-      <c r="J43" s="27"/>
+      <c r="E43" s="19"/>
+      <c r="F43" s="19"/>
+      <c r="G43" s="19"/>
+      <c r="H43" s="19"/>
+      <c r="I43" s="19"/>
+      <c r="J43" s="19"/>
     </row>
     <row r="44" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B44" s="18" t="s">
-        <v>13</v>
-      </c>
-      <c r="C44" s="18">
+      <c r="B44" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="C44" s="12">
         <v>2025</v>
       </c>
-      <c r="D44" s="20">
+      <c r="D44" s="14">
         <v>99.983831740306698</v>
       </c>
-      <c r="E44" s="20">
+      <c r="E44" s="14">
         <v>45.750066254224578</v>
       </c>
-      <c r="F44" s="20">
+      <c r="F44" s="14">
         <v>2.9200234064490638</v>
       </c>
-      <c r="G44" s="20">
+      <c r="G44" s="14">
         <v>27.197595962309034</v>
       </c>
-      <c r="H44" s="20">
+      <c r="H44" s="14">
         <v>19.753893559037373</v>
       </c>
-      <c r="I44" s="20">
+      <c r="I44" s="14">
         <v>0.95617662121596836</v>
       </c>
-      <c r="J44" s="20">
+      <c r="J44" s="14">
         <v>3.4060759370706823</v>
       </c>
     </row>
     <row r="45" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B45" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="C45" s="18">
+      <c r="B45" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C45" s="12">
         <v>2025</v>
       </c>
-      <c r="D45" s="20">
-        <v>96.641120405685058</v>
-      </c>
-      <c r="E45" s="20">
+      <c r="D45" s="14">
+        <v>99.983831740306698</v>
+      </c>
+      <c r="E45" s="14">
         <v>42.066851847558226</v>
       </c>
-      <c r="F45" s="20">
+      <c r="F45" s="14">
         <v>11.631097195887136</v>
       </c>
-      <c r="G45" s="20">
+      <c r="G45" s="14">
         <v>9.633920097542962</v>
       </c>
-      <c r="H45" s="20">
+      <c r="H45" s="14">
         <v>28.744729636147266</v>
       </c>
-      <c r="I45" s="20">
+      <c r="I45" s="14">
         <v>2.6248284734943361</v>
       </c>
-      <c r="J45" s="20">
-        <v>1.9396931550551328</v>
+      <c r="J45" s="14">
+        <v>5.3</v>
       </c>
     </row>
     <row r="46" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B46" s="18" t="s">
-        <v>13</v>
-      </c>
-      <c r="C46" s="18">
+      <c r="B46" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="C46" s="12">
         <v>2024</v>
       </c>
-      <c r="D46" s="20">
+      <c r="D46" s="14">
         <v>100</v>
       </c>
-      <c r="E46" s="20">
+      <c r="E46" s="14">
         <v>45.891590426814751</v>
       </c>
-      <c r="F46" s="20">
+      <c r="F46" s="14">
         <v>2.6736410594184163</v>
       </c>
-      <c r="G46" s="20">
+      <c r="G46" s="14">
         <v>26.981693711390143</v>
       </c>
-      <c r="H46" s="20">
+      <c r="H46" s="14">
         <v>20.105300217527088</v>
       </c>
-      <c r="I46" s="20">
+      <c r="I46" s="14">
         <v>0.99995181923253929</v>
       </c>
-      <c r="J46" s="20">
+      <c r="J46" s="14">
         <v>3.3478227656170723</v>
       </c>
     </row>
     <row r="47" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B47" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="C47" s="18">
+      <c r="B47" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C47" s="12">
         <v>2024</v>
       </c>
-      <c r="D47" s="20">
+      <c r="D47" s="14">
         <v>100</v>
       </c>
-      <c r="E47" s="20">
+      <c r="E47" s="14">
         <v>41.514377790445614</v>
       </c>
-      <c r="F47" s="20">
+      <c r="F47" s="14">
         <v>11.720622961235541</v>
       </c>
-      <c r="G47" s="20">
+      <c r="G47" s="14">
         <v>9.9685365543474447</v>
       </c>
-      <c r="H47" s="20">
+      <c r="H47" s="14">
         <v>28.590190407134049</v>
       </c>
-      <c r="I47" s="20">
+      <c r="I47" s="14">
         <v>2.8942324314151304</v>
       </c>
-      <c r="J47" s="20">
+      <c r="J47" s="14">
         <v>5.3120398554222206</v>
       </c>
     </row>
     <row r="48" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B48" s="18" t="s">
-        <v>13</v>
-      </c>
-      <c r="C48" s="18">
+      <c r="B48" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="C48" s="12">
         <v>2023</v>
       </c>
-      <c r="D48" s="20">
+      <c r="D48" s="14">
         <v>99.999999999999986</v>
       </c>
-      <c r="E48" s="20">
+      <c r="E48" s="14">
         <v>46.18152971562143</v>
       </c>
-      <c r="F48" s="20">
+      <c r="F48" s="14">
         <v>2.6884474629420838</v>
       </c>
-      <c r="G48" s="20">
+      <c r="G48" s="14">
         <v>26.44536656282926</v>
       </c>
-      <c r="H48" s="20">
+      <c r="H48" s="14">
         <v>20.451461711140755</v>
       </c>
-      <c r="I48" s="20">
+      <c r="I48" s="14">
         <v>0.96821048089588013</v>
       </c>
-      <c r="J48" s="20">
+      <c r="J48" s="14">
         <v>3.2649840665705745</v>
       </c>
     </row>
     <row r="49" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B49" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="C49" s="18">
+      <c r="B49" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C49" s="12">
         <v>2023</v>
       </c>
-      <c r="D49" s="20">
+      <c r="D49" s="14">
         <v>100.00000000000003</v>
       </c>
-      <c r="E49" s="20">
+      <c r="E49" s="14">
         <v>40.896844610885324</v>
       </c>
-      <c r="F49" s="20">
+      <c r="F49" s="14">
         <v>12.564587635192066</v>
       </c>
-      <c r="G49" s="20">
+      <c r="G49" s="14">
         <v>9.6449185499984296</v>
       </c>
-      <c r="H49" s="20">
+      <c r="H49" s="14">
         <v>29.608234049737053</v>
       </c>
-      <c r="I49" s="20">
+      <c r="I49" s="14">
         <v>2.4139312013631926</v>
       </c>
-      <c r="J49" s="20">
+      <c r="J49" s="14">
         <v>4.8714839528239455</v>
       </c>
     </row>
     <row r="50" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B50" s="18" t="s">
-        <v>13</v>
-      </c>
-      <c r="C50" s="18">
+      <c r="B50" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="C50" s="12">
         <v>2022</v>
       </c>
-      <c r="D50" s="20">
+      <c r="D50" s="14">
         <v>99.999999999999972</v>
       </c>
-      <c r="E50" s="20">
+      <c r="E50" s="14">
         <v>45.590827537329879</v>
       </c>
-      <c r="F50" s="20">
+      <c r="F50" s="14">
         <v>2.6224874852971372</v>
       </c>
-      <c r="G50" s="20">
+      <c r="G50" s="14">
         <v>26.514802963499694</v>
       </c>
-      <c r="H50" s="20">
+      <c r="H50" s="14">
         <v>20.846099243226394</v>
       </c>
-      <c r="I50" s="20">
+      <c r="I50" s="14">
         <v>0.81146467658260824</v>
       </c>
-      <c r="J50" s="20">
+      <c r="J50" s="14">
         <v>3.6143180940642781</v>
       </c>
     </row>
     <row r="51" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B51" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="C51" s="18">
+      <c r="B51" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C51" s="12">
         <v>2022</v>
       </c>
-      <c r="D51" s="20">
+      <c r="D51" s="14">
         <v>100</v>
       </c>
-      <c r="E51" s="20">
+      <c r="E51" s="14">
         <v>41.641959896718333</v>
       </c>
-      <c r="F51" s="20">
+      <c r="F51" s="14">
         <v>10.248653849217144</v>
       </c>
-      <c r="G51" s="20">
+      <c r="G51" s="14">
         <v>9.7749873639676625</v>
       </c>
-      <c r="H51" s="20">
+      <c r="H51" s="14">
         <v>31.735882702153063</v>
       </c>
-      <c r="I51" s="20">
+      <c r="I51" s="14">
         <v>2.2133944855932262</v>
       </c>
-      <c r="J51" s="20">
+      <c r="J51" s="14">
         <v>4.3851217023505757</v>
       </c>
     </row>
     <row r="52" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B52" s="18" t="s">
-        <v>13</v>
-      </c>
-      <c r="C52" s="18">
+      <c r="B52" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="C52" s="12">
         <v>2021</v>
       </c>
-      <c r="D52" s="20">
+      <c r="D52" s="14">
         <v>100</v>
       </c>
-      <c r="E52" s="20">
+      <c r="E52" s="14">
         <v>45.578577881728819</v>
       </c>
-      <c r="F52" s="20">
+      <c r="F52" s="14">
         <v>2.6545559747249889</v>
       </c>
-      <c r="G52" s="20">
+      <c r="G52" s="14">
         <v>26.222618348896837</v>
       </c>
-      <c r="H52" s="20">
+      <c r="H52" s="14">
         <v>21.200706832180423</v>
       </c>
-      <c r="I52" s="20">
+      <c r="I52" s="14">
         <v>0.82754448113808976</v>
       </c>
-      <c r="J52" s="20">
+      <c r="J52" s="14">
         <v>3.5159964813308702</v>
       </c>
     </row>
     <row r="53" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B53" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="C53" s="18">
+      <c r="B53" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C53" s="12">
         <v>2021</v>
       </c>
-      <c r="D53" s="20">
+      <c r="D53" s="14">
         <v>100</v>
       </c>
-      <c r="E53" s="20">
+      <c r="E53" s="14">
         <v>40.939157323737348</v>
       </c>
-      <c r="F53" s="20">
+      <c r="F53" s="14">
         <v>9.091370465361944</v>
       </c>
-      <c r="G53" s="20">
+      <c r="G53" s="14">
         <v>10.556154326779152</v>
       </c>
-      <c r="H53" s="20">
+      <c r="H53" s="14">
         <v>33.042990358118033</v>
       </c>
-      <c r="I53" s="20">
+      <c r="I53" s="14">
         <v>1.8766205979873476</v>
       </c>
-      <c r="J53" s="20">
+      <c r="J53" s="14">
         <v>4.4937069280161888</v>
       </c>
     </row>
     <row r="54" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B54" s="18" t="s">
-        <v>13</v>
-      </c>
-      <c r="C54" s="18">
+      <c r="B54" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="C54" s="12">
         <v>2020</v>
       </c>
-      <c r="D54" s="20">
+      <c r="D54" s="14">
         <v>99.999999999999986</v>
       </c>
-      <c r="E54" s="20">
+      <c r="E54" s="14">
         <v>47.187141216991961</v>
       </c>
-      <c r="F54" s="20">
+      <c r="F54" s="14">
         <v>2.1485976709857306</v>
       </c>
-      <c r="G54" s="20">
+      <c r="G54" s="14">
         <v>26.832868623913399</v>
       </c>
-      <c r="H54" s="20">
+      <c r="H54" s="14">
         <v>19.763818271280957</v>
       </c>
-      <c r="I54" s="20">
+      <c r="I54" s="14">
         <v>0.63965884861407252</v>
       </c>
-      <c r="J54" s="20">
+      <c r="J54" s="14">
         <v>3.4279153682138754</v>
       </c>
     </row>
     <row r="55" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B55" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="C55" s="18">
+      <c r="B55" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C55" s="12">
         <v>2020</v>
       </c>
-      <c r="D55" s="20">
+      <c r="D55" s="14">
         <v>100</v>
       </c>
-      <c r="E55" s="20">
+      <c r="E55" s="14">
         <v>42.269187986651836</v>
       </c>
-      <c r="F55" s="20">
+      <c r="F55" s="14">
         <v>9.3993325917686317</v>
       </c>
-      <c r="G55" s="20">
+      <c r="G55" s="14">
         <v>9.788654060066742</v>
       </c>
-      <c r="H55" s="20">
+      <c r="H55" s="14">
         <v>30.42269187986652</v>
       </c>
-      <c r="I55" s="20">
+      <c r="I55" s="14">
         <v>2.2803114571746388</v>
       </c>
-      <c r="J55" s="20">
+      <c r="J55" s="14">
         <v>5.8398220244716352</v>
       </c>
     </row>
     <row r="56" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B56" s="18" t="s">
-        <v>13</v>
-      </c>
-      <c r="C56" s="18">
+      <c r="B56" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="C56" s="12">
         <v>2019</v>
       </c>
-      <c r="D56" s="20">
+      <c r="D56" s="14">
         <v>100</v>
       </c>
-      <c r="E56" s="20">
+      <c r="E56" s="14">
         <v>47.131973457852048</v>
       </c>
-      <c r="F56" s="20">
+      <c r="F56" s="14">
         <v>2.464159908249365</v>
       </c>
-      <c r="G56" s="20">
+      <c r="G56" s="14">
         <v>25.142950765953959</v>
       </c>
-      <c r="H56" s="20">
+      <c r="H56" s="14">
         <v>22.321618743343986</v>
       </c>
-      <c r="I56" s="20">
+      <c r="I56" s="14">
         <v>0.63897763578274758</v>
       </c>
-      <c r="J56" s="20">
+      <c r="J56" s="14">
         <v>2.3003194888178915</v>
       </c>
     </row>
     <row r="57" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B57" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="C57" s="18">
+      <c r="B57" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C57" s="12">
         <v>2019</v>
       </c>
-      <c r="D57" s="20">
+      <c r="D57" s="14">
         <v>100</v>
       </c>
-      <c r="E57" s="20">
+      <c r="E57" s="14">
         <v>40.735557545902374</v>
       </c>
-      <c r="F57" s="20">
+      <c r="F57" s="14">
         <v>7.5850873264666356</v>
       </c>
-      <c r="G57" s="20">
+      <c r="G57" s="14">
         <v>9.3652037617554864</v>
       </c>
-      <c r="H57" s="20">
+      <c r="H57" s="14">
         <v>35.031347962382441</v>
       </c>
-      <c r="I57" s="20">
+      <c r="I57" s="14">
         <v>2.2503358710255261</v>
       </c>
-      <c r="J57" s="20">
+      <c r="J57" s="14">
         <v>5.0324675324675328</v>
       </c>
     </row>
     <row r="58" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B58" s="18" t="s">
-        <v>13</v>
-      </c>
-      <c r="C58" s="18">
+      <c r="B58" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="C58" s="12">
         <v>2018</v>
       </c>
-      <c r="D58" s="20">
+      <c r="D58" s="14">
         <v>100.00000000000001</v>
       </c>
-      <c r="E58" s="20">
+      <c r="E58" s="14">
         <v>46.405292980904655</v>
       </c>
-      <c r="F58" s="20">
+      <c r="F58" s="14">
         <v>2.5498673479414364</v>
       </c>
-      <c r="G58" s="20">
+      <c r="G58" s="14">
         <v>25.198978087845141</v>
       </c>
-      <c r="H58" s="20">
+      <c r="H58" s="14">
         <v>23.017588680357669</v>
       </c>
-      <c r="I58" s="20">
+      <c r="I58" s="14">
         <v>0.52078215584160359</v>
       </c>
-      <c r="J58" s="20">
+      <c r="J58" s="14">
         <v>2.3074907471094952</v>
       </c>
     </row>
     <row r="59" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B59" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="C59" s="18">
+      <c r="B59" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C59" s="12">
         <v>2018</v>
       </c>
-      <c r="D59" s="20">
+      <c r="D59" s="14">
         <v>100</v>
       </c>
-      <c r="E59" s="20">
+      <c r="E59" s="14">
         <v>40.487140180548451</v>
       </c>
-      <c r="F59" s="20">
+      <c r="F59" s="14">
         <v>7.6307273036961334</v>
       </c>
-      <c r="G59" s="20">
+      <c r="G59" s="14">
         <v>9.0387781752114904</v>
       </c>
-      <c r="H59" s="20">
+      <c r="H59" s="14">
         <v>35.439732016124452</v>
       </c>
-      <c r="I59" s="20">
+      <c r="I59" s="14">
         <v>2.3221484131039567</v>
       </c>
-      <c r="J59" s="20">
+      <c r="J59" s="14">
         <v>5.0814739113155056</v>
       </c>
     </row>
     <row r="60" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B60" s="18" t="s">
-        <v>13</v>
-      </c>
-      <c r="C60" s="18">
+      <c r="B60" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="C60" s="12">
         <v>2017</v>
       </c>
-      <c r="D60" s="20">
+      <c r="D60" s="14">
         <v>100</v>
       </c>
-      <c r="E60" s="20">
+      <c r="E60" s="14">
         <v>46.073550666452547</v>
       </c>
-      <c r="F60" s="20">
+      <c r="F60" s="14">
         <v>2.6336919865103581</v>
       </c>
-      <c r="G60" s="20">
+      <c r="G60" s="14">
         <v>24.32953268026337</v>
       </c>
-      <c r="H60" s="20">
+      <c r="H60" s="14">
         <v>23.301750441625181</v>
       </c>
-      <c r="I60" s="20">
+      <c r="I60" s="14">
         <v>0.69054119158503291</v>
       </c>
-      <c r="J60" s="20">
+      <c r="J60" s="14">
         <v>2.9709330335635138</v>
       </c>
     </row>
     <row r="61" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B61" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="C61" s="18">
+      <c r="B61" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C61" s="12">
         <v>2017</v>
       </c>
-      <c r="D61" s="20">
+      <c r="D61" s="14">
         <v>100</v>
       </c>
-      <c r="E61" s="20">
+      <c r="E61" s="14">
         <v>37.742504409171076</v>
       </c>
-      <c r="F61" s="20">
+      <c r="F61" s="14">
         <v>7.2310405643738971</v>
       </c>
-      <c r="G61" s="20">
+      <c r="G61" s="14">
         <v>9.4062316284538507</v>
       </c>
-      <c r="H61" s="20">
+      <c r="H61" s="14">
         <v>35.978835978835974</v>
       </c>
-      <c r="I61" s="20">
+      <c r="I61" s="14">
         <v>2.7042915931804821</v>
       </c>
-      <c r="J61" s="20">
+      <c r="J61" s="14">
         <v>6.9370958259847155</v>
       </c>
     </row>
     <row r="62" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B62" s="18" t="s">
-        <v>13</v>
-      </c>
-      <c r="C62" s="18">
+      <c r="B62" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="C62" s="12">
         <v>2016</v>
       </c>
-      <c r="D62" s="20">
+      <c r="D62" s="14">
         <v>100</v>
       </c>
-      <c r="E62" s="20">
+      <c r="E62" s="14">
         <v>45.022659790592279</v>
       </c>
-      <c r="F62" s="20">
+      <c r="F62" s="14">
         <v>2.7816846382247227</v>
       </c>
-      <c r="G62" s="20">
+      <c r="G62" s="14">
         <v>24.894514767932492</v>
       </c>
-      <c r="H62" s="20">
+      <c r="H62" s="14">
         <v>24.175652445694638</v>
       </c>
-      <c r="I62" s="20">
+      <c r="I62" s="14">
         <v>0.96890139084231908</v>
       </c>
-      <c r="J62" s="20">
+      <c r="J62" s="14">
         <v>2.1565869667135491</v>
       </c>
     </row>
     <row r="63" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B63" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="C63" s="18">
+      <c r="B63" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C63" s="12">
         <v>2016</v>
       </c>
-      <c r="D63" s="20">
+      <c r="D63" s="14">
         <v>100</v>
       </c>
-      <c r="E63" s="20">
+      <c r="E63" s="14">
         <v>37.264742785445421</v>
       </c>
-      <c r="F63" s="20">
+      <c r="F63" s="14">
         <v>6.7754077791718954</v>
       </c>
-      <c r="G63" s="20">
+      <c r="G63" s="14">
         <v>9.5357590966122974</v>
       </c>
-      <c r="H63" s="20">
+      <c r="H63" s="14">
         <v>36.700125470514429</v>
       </c>
-      <c r="I63" s="20">
+      <c r="I63" s="14">
         <v>3.4504391468005018</v>
       </c>
-      <c r="J63" s="20">
+      <c r="J63" s="14">
         <v>6.2735257214554583</v>
       </c>
     </row>
     <row r="64" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B64" s="18" t="s">
-        <v>13</v>
-      </c>
-      <c r="C64" s="18">
+      <c r="B64" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="C64" s="12">
         <v>2015</v>
       </c>
-      <c r="D64" s="20">
+      <c r="D64" s="14">
         <v>100</v>
       </c>
-      <c r="E64" s="20">
+      <c r="E64" s="14">
         <v>44.339476537091528</v>
       </c>
-      <c r="F64" s="20">
+      <c r="F64" s="14">
         <v>3.1283877961901809</v>
       </c>
-      <c r="G64" s="20">
+      <c r="G64" s="14">
         <v>24.903205823137682</v>
       </c>
-      <c r="H64" s="20">
+      <c r="H64" s="14">
         <v>24.639925662072169</v>
       </c>
-      <c r="I64" s="20">
+      <c r="I64" s="14">
         <v>0.83630168809044436</v>
       </c>
-      <c r="J64" s="20">
+      <c r="J64" s="14">
         <v>2.1527024934179959</v>
       </c>
     </row>
     <row r="65" spans="1:13" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B65" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="C65" s="18">
+      <c r="B65" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C65" s="12">
         <v>2015</v>
       </c>
-      <c r="D65" s="20">
+      <c r="D65" s="14">
         <v>100</v>
       </c>
-      <c r="E65" s="20">
+      <c r="E65" s="14">
         <v>37.784090909090914</v>
       </c>
-      <c r="F65" s="20">
+      <c r="F65" s="14">
         <v>7.9545454545454541</v>
       </c>
-      <c r="G65" s="20">
+      <c r="G65" s="14">
         <v>10.15625</v>
       </c>
-      <c r="H65" s="20">
+      <c r="H65" s="14">
         <v>38.352272727272727</v>
       </c>
-      <c r="I65" s="20">
+      <c r="I65" s="14">
         <v>2.8409090909090908</v>
       </c>
-      <c r="J65" s="20">
+      <c r="J65" s="14">
         <v>2.9119318181818179</v>
       </c>
     </row>
     <row r="66" spans="1:13" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B66" s="18" t="s">
-        <v>13</v>
-      </c>
-      <c r="C66" s="18">
+      <c r="B66" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="C66" s="12">
         <v>2014</v>
       </c>
-      <c r="D66" s="20">
+      <c r="D66" s="14">
         <v>100</v>
       </c>
-      <c r="E66" s="20">
+      <c r="E66" s="14">
         <v>43.86374241717219</v>
       </c>
-      <c r="F66" s="20">
+      <c r="F66" s="14">
         <v>3.282003421994089</v>
       </c>
-      <c r="G66" s="20">
+      <c r="G66" s="14">
         <v>24.498366775548298</v>
       </c>
-      <c r="H66" s="20">
+      <c r="H66" s="14">
         <v>25.773837299735575</v>
       </c>
-      <c r="I66" s="20">
+      <c r="I66" s="14">
         <v>0.9643801524342821</v>
       </c>
-      <c r="J66" s="20">
+      <c r="J66" s="14">
         <v>1.6176699331155699</v>
       </c>
     </row>
     <row r="67" spans="1:13" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B67" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="C67" s="18">
+      <c r="B67" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C67" s="12">
         <v>2014</v>
       </c>
-      <c r="D67" s="20">
+      <c r="D67" s="14">
         <v>100.00000000000001</v>
       </c>
-      <c r="E67" s="20">
+      <c r="E67" s="14">
         <v>38.179148311306903</v>
       </c>
-      <c r="F67" s="20">
+      <c r="F67" s="14">
         <v>7.2687224669603516</v>
       </c>
-      <c r="G67" s="20">
+      <c r="G67" s="14">
         <v>10.279001468428781</v>
       </c>
-      <c r="H67" s="20">
+      <c r="H67" s="14">
         <v>40.161527165932455</v>
       </c>
-      <c r="I67" s="20">
+      <c r="I67" s="14">
         <v>2.2026431718061676</v>
       </c>
-      <c r="J67" s="20">
+      <c r="J67" s="14">
         <v>1.908957415565345</v>
       </c>
     </row>
     <row r="68" spans="1:13" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B68" s="18" t="s">
-        <v>13</v>
-      </c>
-      <c r="C68" s="18">
+      <c r="B68" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="C68" s="12">
         <v>2013</v>
       </c>
-      <c r="D68" s="20">
+      <c r="D68" s="14">
         <v>100</v>
       </c>
-      <c r="E68" s="20">
+      <c r="E68" s="14">
         <v>43.32339557508238</v>
       </c>
-      <c r="F68" s="20">
+      <c r="F68" s="14">
         <v>3.3108426172916996</v>
       </c>
-      <c r="G68" s="20">
+      <c r="G68" s="14">
         <v>24.80778283383022</v>
       </c>
-      <c r="H68" s="20">
+      <c r="H68" s="14">
         <v>26.408284952141848</v>
       </c>
-      <c r="I68" s="20">
+      <c r="I68" s="14">
         <v>0.70610387572571787</v>
       </c>
-      <c r="J68" s="20">
+      <c r="J68" s="14">
         <v>1.4435901459281344</v>
       </c>
     </row>
     <row r="69" spans="1:13" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B69" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="C69" s="18">
+      <c r="B69" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C69" s="12">
         <v>2013</v>
       </c>
-      <c r="D69" s="20">
+      <c r="D69" s="14">
         <v>100</v>
       </c>
-      <c r="E69" s="20">
+      <c r="E69" s="14">
         <v>39.034776437189493</v>
       </c>
-      <c r="F69" s="20">
+      <c r="F69" s="14">
         <v>7.8069552874378987</v>
       </c>
-      <c r="G69" s="20">
+      <c r="G69" s="14">
         <v>9.7232079488999279</v>
       </c>
-      <c r="H69" s="20">
+      <c r="H69" s="14">
         <v>39.531582682753722</v>
       </c>
-      <c r="I69" s="20">
+      <c r="I69" s="14">
         <v>1.7743080198722498</v>
       </c>
-      <c r="J69" s="20">
+      <c r="J69" s="14">
         <v>2.1291696238466997</v>
       </c>
     </row>
     <row r="70" spans="1:13" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B70" s="18" t="s">
-        <v>13</v>
-      </c>
-      <c r="C70" s="18">
+      <c r="B70" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="C70" s="12">
         <v>2012</v>
       </c>
-      <c r="D70" s="20">
+      <c r="D70" s="14">
         <v>100</v>
       </c>
-      <c r="E70" s="20">
+      <c r="E70" s="14">
         <v>42.942989214175654</v>
       </c>
-      <c r="F70" s="20">
+      <c r="F70" s="14">
         <v>3.2973805855161791</v>
       </c>
-      <c r="G70" s="20">
+      <c r="G70" s="14">
         <v>24.298921417565484</v>
       </c>
-      <c r="H70" s="20">
+      <c r="H70" s="14">
         <v>26.610169491525426</v>
       </c>
-      <c r="I70" s="20">
+      <c r="I70" s="14">
         <v>0.75500770416024654</v>
       </c>
-      <c r="J70" s="20">
+      <c r="J70" s="14">
         <v>2.0955315870570108</v>
       </c>
     </row>
     <row r="71" spans="1:13" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B71" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="C71" s="18">
+      <c r="B71" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C71" s="12">
         <v>2012</v>
       </c>
-      <c r="D71" s="20">
+      <c r="D71" s="14">
         <v>100</v>
       </c>
-      <c r="E71" s="20">
+      <c r="E71" s="14">
         <v>37.223493516399699</v>
       </c>
-      <c r="F71" s="20">
+      <c r="F71" s="14">
         <v>7.8565980167810832</v>
       </c>
-      <c r="G71" s="20">
+      <c r="G71" s="14">
         <v>9.9923722349351642</v>
       </c>
-      <c r="H71" s="20">
+      <c r="H71" s="14">
         <v>40.274599542334094</v>
       </c>
-      <c r="I71" s="20">
+      <c r="I71" s="14">
         <v>1.9069412662090008</v>
       </c>
-      <c r="J71" s="20">
+      <c r="J71" s="14">
         <v>2.7459954233409611</v>
       </c>
     </row>
     <row r="72" spans="1:13" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B72" s="18" t="s">
-        <v>13</v>
-      </c>
-      <c r="C72" s="18">
+      <c r="B72" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="C72" s="12">
         <v>2011</v>
       </c>
-      <c r="D72" s="20">
+      <c r="D72" s="14">
         <v>100</v>
       </c>
-      <c r="E72" s="20">
+      <c r="E72" s="14">
         <v>42.87248734080098</v>
       </c>
-      <c r="F72" s="20">
+      <c r="F72" s="14">
         <v>3.5599202086849782</v>
       </c>
-      <c r="G72" s="20">
+      <c r="G72" s="14">
         <v>24.443762467392972</v>
       </c>
-      <c r="H72" s="20">
+      <c r="H72" s="14">
         <v>26.300444990026083</v>
       </c>
-      <c r="I72" s="20">
+      <c r="I72" s="14">
         <v>0.78256866656437019</v>
       </c>
-      <c r="J72" s="20">
+      <c r="J72" s="14">
         <v>2.0408163265306123</v>
       </c>
     </row>
     <row r="73" spans="1:13" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B73" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="C73" s="18">
+      <c r="B73" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C73" s="12">
         <v>2011</v>
       </c>
-      <c r="D73" s="20">
+      <c r="D73" s="14">
         <v>100</v>
       </c>
-      <c r="E73" s="20">
+      <c r="E73" s="14">
         <v>37.156323644933231</v>
       </c>
-      <c r="F73" s="20">
+      <c r="F73" s="14">
         <v>8.7981146897093474</v>
       </c>
-      <c r="G73" s="20">
+      <c r="G73" s="14">
         <v>9.8978790259230163</v>
       </c>
-      <c r="H73" s="20">
+      <c r="H73" s="14">
         <v>39.591516103692065</v>
       </c>
-      <c r="I73" s="20">
+      <c r="I73" s="14">
         <v>2.1995286724273369</v>
       </c>
-      <c r="J73" s="20">
+      <c r="J73" s="14">
         <v>2.356637863315004</v>
       </c>
     </row>
     <row r="74" spans="1:13" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A74" s="10"/>
-      <c r="B74" s="13"/>
-      <c r="C74" s="14"/>
-      <c r="D74" s="14"/>
-      <c r="E74" s="14"/>
-      <c r="F74" s="14"/>
-      <c r="G74" s="14"/>
-      <c r="H74" s="14"/>
-      <c r="I74" s="10"/>
-      <c r="J74" s="10"/>
-      <c r="K74" s="10"/>
-      <c r="L74" s="10"/>
-      <c r="M74" s="10"/>
-    </row>
-    <row r="75" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A74" s="9"/>
+      <c r="B74" s="10"/>
+      <c r="C74" s="11"/>
+      <c r="D74" s="11"/>
+      <c r="E74" s="11"/>
+      <c r="F74" s="11"/>
+      <c r="G74" s="11"/>
+      <c r="H74" s="11"/>
+      <c r="I74" s="9"/>
+      <c r="J74" s="9"/>
+      <c r="K74" s="9"/>
+      <c r="L74" s="9"/>
+      <c r="M74" s="9"/>
+    </row>
+    <row r="75" spans="1:13" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A75" s="8"/>
-      <c r="B75" s="21" t="s">
+      <c r="B75" s="20" t="s">
+        <v>22</v>
+      </c>
+      <c r="C75" s="20"/>
+      <c r="D75" s="20"/>
+      <c r="E75" s="20"/>
+      <c r="F75" s="20"/>
+      <c r="G75" s="20"/>
+      <c r="H75" s="20"/>
+      <c r="I75" s="20"/>
+      <c r="J75" s="20"/>
+      <c r="K75" s="20"/>
+      <c r="L75" s="20"/>
+      <c r="M75" s="20"/>
+    </row>
+    <row r="76" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A76" s="9"/>
+      <c r="B76" s="20" t="s">
+        <v>23</v>
+      </c>
+      <c r="C76" s="20"/>
+      <c r="D76" s="20"/>
+      <c r="E76" s="20"/>
+      <c r="F76" s="20"/>
+      <c r="G76" s="20"/>
+      <c r="H76" s="20"/>
+      <c r="I76" s="20"/>
+      <c r="J76" s="20"/>
+      <c r="K76" s="20"/>
+      <c r="L76" s="20"/>
+      <c r="M76" s="20"/>
+    </row>
+    <row r="77" spans="1:13" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A77" s="9"/>
+      <c r="B77" s="20" t="s">
+        <v>24</v>
+      </c>
+      <c r="C77" s="20"/>
+      <c r="D77" s="20"/>
+      <c r="E77" s="20"/>
+      <c r="F77" s="20"/>
+      <c r="G77" s="20"/>
+      <c r="H77" s="20"/>
+      <c r="I77" s="20"/>
+      <c r="J77" s="20"/>
+      <c r="K77" s="20"/>
+      <c r="L77" s="20"/>
+      <c r="M77" s="20"/>
+    </row>
+    <row r="78" spans="1:13" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A78" s="9"/>
+      <c r="B78" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="C75" s="21"/>
-      <c r="D75" s="21"/>
-      <c r="E75" s="21"/>
-      <c r="F75" s="21"/>
-      <c r="G75" s="21"/>
-      <c r="H75" s="21"/>
-      <c r="I75" s="21"/>
-      <c r="J75" s="21"/>
-      <c r="K75" s="9"/>
-      <c r="L75" s="9"/>
-      <c r="M75" s="9"/>
-    </row>
-    <row r="76" spans="1:13" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A76" s="10"/>
-      <c r="B76" s="11" t="s">
+      <c r="C78" s="22"/>
+      <c r="D78" s="22"/>
+      <c r="E78" s="22"/>
+      <c r="F78" s="22"/>
+      <c r="G78" s="22"/>
+      <c r="H78" s="22"/>
+      <c r="I78" s="22"/>
+      <c r="J78" s="22"/>
+      <c r="K78" s="22"/>
+      <c r="L78" s="22"/>
+      <c r="M78" s="22"/>
+    </row>
+    <row r="79" spans="1:13" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A79" s="9"/>
+      <c r="B79" s="21"/>
+      <c r="C79" s="22"/>
+      <c r="D79" s="22"/>
+      <c r="E79" s="22"/>
+      <c r="F79" s="22"/>
+      <c r="G79" s="22"/>
+      <c r="H79" s="22"/>
+      <c r="I79" s="22"/>
+      <c r="J79" s="22"/>
+      <c r="K79" s="22"/>
+      <c r="L79" s="22"/>
+      <c r="M79" s="22"/>
+    </row>
+    <row r="80" spans="1:13" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B80" s="23" t="s">
         <v>17</v>
       </c>
-      <c r="C76" s="10"/>
-      <c r="D76" s="10"/>
-      <c r="E76" s="10"/>
-      <c r="F76" s="10"/>
-      <c r="G76" s="10"/>
-      <c r="H76" s="10"/>
-      <c r="I76" s="10"/>
-      <c r="J76" s="10"/>
-      <c r="K76" s="10"/>
-      <c r="L76" s="10"/>
-      <c r="M76" s="10"/>
-    </row>
-    <row r="77" spans="1:13" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A77" s="10"/>
-      <c r="B77" s="22" t="s">
+      <c r="C80" s="22"/>
+      <c r="D80" s="22"/>
+      <c r="E80" s="22"/>
+      <c r="F80" s="22"/>
+      <c r="G80" s="22"/>
+      <c r="H80" s="22"/>
+      <c r="I80" s="22"/>
+      <c r="J80" s="22"/>
+      <c r="K80" s="22"/>
+      <c r="L80" s="22"/>
+      <c r="M80" s="22"/>
+    </row>
+    <row r="81" spans="2:13" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B81" s="22"/>
+      <c r="C81" s="22"/>
+      <c r="D81" s="22"/>
+      <c r="E81" s="22"/>
+      <c r="F81" s="22"/>
+      <c r="G81" s="22"/>
+      <c r="H81" s="22"/>
+      <c r="I81" s="22"/>
+      <c r="J81" s="22"/>
+      <c r="K81" s="22"/>
+      <c r="L81" s="22"/>
+      <c r="M81" s="22"/>
+    </row>
+    <row r="82" spans="2:13" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B82" s="24" t="s">
         <v>18</v>
       </c>
-      <c r="C77" s="22"/>
-      <c r="D77" s="22"/>
-      <c r="E77" s="22"/>
-      <c r="F77" s="22"/>
-      <c r="G77" s="22"/>
-      <c r="H77" s="22"/>
-      <c r="I77" s="22"/>
-      <c r="J77" s="22"/>
-      <c r="K77" s="12"/>
-      <c r="L77" s="12"/>
-      <c r="M77" s="12"/>
-    </row>
-    <row r="78" spans="1:13" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A78" s="10"/>
-      <c r="B78" s="13" t="s">
+      <c r="C82" s="22"/>
+      <c r="D82" s="22"/>
+      <c r="E82" s="22"/>
+      <c r="F82" s="22"/>
+      <c r="G82" s="22"/>
+      <c r="H82" s="22"/>
+      <c r="I82" s="22"/>
+      <c r="J82" s="22"/>
+      <c r="K82" s="22"/>
+      <c r="L82" s="22"/>
+      <c r="M82" s="22"/>
+    </row>
+    <row r="83" spans="2:13" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B83" s="24" t="s">
+        <v>25</v>
+      </c>
+      <c r="C83" s="22"/>
+      <c r="D83" s="22"/>
+      <c r="E83" s="22"/>
+      <c r="F83" s="22"/>
+      <c r="G83" s="22"/>
+      <c r="H83" s="22"/>
+      <c r="I83" s="22"/>
+      <c r="J83" s="22"/>
+      <c r="K83" s="22"/>
+      <c r="L83" s="22"/>
+      <c r="M83" s="22"/>
+    </row>
+    <row r="84" spans="2:13" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B84" s="24" t="s">
         <v>19</v>
       </c>
-      <c r="C78" s="14"/>
-      <c r="D78" s="14"/>
-      <c r="E78" s="14"/>
-      <c r="F78" s="14"/>
-      <c r="G78" s="14"/>
-      <c r="H78" s="14"/>
-      <c r="I78" s="10"/>
-      <c r="J78" s="10"/>
-      <c r="K78" s="10"/>
-      <c r="L78" s="10"/>
-      <c r="M78" s="10"/>
-    </row>
-    <row r="79" spans="1:13" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A79" s="10"/>
-      <c r="B79" s="14"/>
-      <c r="C79" s="14"/>
-      <c r="D79" s="14"/>
-      <c r="E79" s="14"/>
-      <c r="F79" s="14"/>
-      <c r="G79" s="14"/>
-      <c r="H79" s="14"/>
-      <c r="I79" s="10"/>
-      <c r="J79" s="10"/>
-      <c r="K79" s="10"/>
-      <c r="L79" s="10"/>
-      <c r="M79" s="10"/>
-    </row>
-    <row r="80" spans="1:13" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B80" s="11" t="s">
+      <c r="C84" s="22"/>
+      <c r="D84" s="22"/>
+      <c r="E84" s="22"/>
+      <c r="F84" s="22"/>
+      <c r="G84" s="22"/>
+      <c r="H84" s="22"/>
+      <c r="I84" s="22"/>
+      <c r="J84" s="22"/>
+      <c r="K84" s="22"/>
+      <c r="L84" s="22"/>
+      <c r="M84" s="22"/>
+    </row>
+    <row r="85" spans="2:13" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B85" s="25" t="s">
         <v>20</v>
       </c>
-      <c r="C80" s="15"/>
-      <c r="D80" s="15"/>
-      <c r="E80" s="15"/>
-      <c r="F80" s="16"/>
-      <c r="G80" s="16"/>
-      <c r="H80" s="10"/>
-    </row>
-    <row r="81" spans="2:8" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B81" s="10"/>
-      <c r="C81" s="10"/>
-      <c r="D81" s="10"/>
-      <c r="E81" s="10"/>
-      <c r="F81" s="10"/>
-      <c r="G81" s="10"/>
-      <c r="H81" s="10"/>
-    </row>
-    <row r="82" spans="2:8" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B82" s="11" t="s">
-        <v>21</v>
-      </c>
-      <c r="C82" s="10"/>
-      <c r="D82" s="10"/>
-      <c r="E82" s="10"/>
-      <c r="F82" s="10"/>
-      <c r="G82" s="10"/>
-      <c r="H82" s="10"/>
-    </row>
-    <row r="83" spans="2:8" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B83" s="11" t="s">
-        <v>25</v>
-      </c>
-      <c r="C83" s="10"/>
-      <c r="D83" s="10"/>
-      <c r="E83" s="10"/>
-      <c r="F83" s="10"/>
-      <c r="G83" s="10"/>
-      <c r="H83" s="10"/>
-    </row>
-    <row r="84" spans="2:8" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B84" s="11" t="s">
-        <v>22</v>
-      </c>
-      <c r="C84" s="10"/>
-      <c r="D84" s="10"/>
-      <c r="E84" s="10"/>
-      <c r="F84" s="10"/>
-      <c r="G84" s="10"/>
-      <c r="H84" s="10"/>
-    </row>
-    <row r="85" spans="2:8" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B85" s="17" t="s">
-        <v>23</v>
-      </c>
-      <c r="C85" s="10"/>
-      <c r="D85" s="10"/>
-      <c r="E85" s="10"/>
-      <c r="F85" s="10"/>
-      <c r="G85" s="10"/>
-      <c r="H85" s="10"/>
+      <c r="C85" s="22"/>
+      <c r="D85" s="22"/>
+      <c r="E85" s="22"/>
+      <c r="F85" s="22"/>
+      <c r="G85" s="22"/>
+      <c r="H85" s="22"/>
+      <c r="I85" s="22"/>
+      <c r="J85" s="22"/>
+      <c r="K85" s="22"/>
+      <c r="L85" s="22"/>
+      <c r="M85" s="22"/>
     </row>
   </sheetData>
-  <mergeCells count="10">
+  <mergeCells count="11">
+    <mergeCell ref="B41:B43"/>
+    <mergeCell ref="C41:C43"/>
+    <mergeCell ref="D41:J41"/>
+    <mergeCell ref="D43:J43"/>
+    <mergeCell ref="B75:M75"/>
+    <mergeCell ref="B76:M76"/>
+    <mergeCell ref="B77:M77"/>
     <mergeCell ref="B6:B8"/>
     <mergeCell ref="C6:C8"/>
     <mergeCell ref="D6:J6"/>
     <mergeCell ref="D8:J8"/>
-    <mergeCell ref="B75:J75"/>
-    <mergeCell ref="B77:J77"/>
-    <mergeCell ref="B41:B43"/>
-    <mergeCell ref="C41:C43"/>
-    <mergeCell ref="D41:J41"/>
-    <mergeCell ref="D43:J43"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="B85" r:id="rId1" xr:uid="{E8296B3C-0891-4298-B260-2E9053746E12}"/>
-    <hyperlink ref="B78" r:id="rId2" xr:uid="{C5DE47B4-1D36-4837-95AA-46AE8069022F}"/>
+    <hyperlink ref="B78" r:id="rId1" xr:uid="{E99B2DBB-3654-48CF-894B-543051D83AA2}"/>
+    <hyperlink ref="B85" r:id="rId2" xr:uid="{F4662E07-0D12-46BB-802C-845C04E86A33}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Deploying to gh-pages from  @ 9f803969a2a14222baa75a52ebd4430a0b94c558 🚀
</commit_message>
<xml_diff>
--- a/assets/excel/2026_6-3-1.xlsx
+++ b/assets/excel/2026_6-3-1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr codeName="DieseArbeitsmappe" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\Hannover\Dez15_Uebergreifende_Analysen\Projekte\Integrationsmonitoring\Schlesier\MT_Site\assets\excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\BiesterChristophLSN\Desktop\MZ\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32CF31D2-5072-4EDF-B983-268934BDB332}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{EED34A05-2686-4678-9FA0-CD53D7D61E19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{26AA0D46-F1BF-4408-A6F5-D4E9B3798D9B}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15270" xr2:uid="{26AA0D46-F1BF-4408-A6F5-D4E9B3798D9B}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="2" r:id="rId1"/>
@@ -104,15 +104,6 @@
     <t>Prozent</t>
   </si>
   <si>
-    <t>1) Seit dem Jahr 2018 wird im Mikrozensus der Migrationshintergrund im weiteren Sinne jährlich berichtet. Die in der Tabelle ab dem Jahr 2018 abgebildeten Daten zum Migrationshintergrund entsprechen dem Migrationshintergrund im weiteren Sinne, bis 2017 wird der Migrationshintergrund im engeren Sinne abgebildet. Die Vergleichbarkeit ist dadurch eingeschränkt.</t>
-  </si>
-  <si>
-    <t>2) Einschl. Grundsicherung im Alter und bei Erwerbsminderung und andere Hilfen in besonderen Lebenslagen.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3) Die Ergebnisse des Mikrozensus 2020 sind unter anderem aufgrund methodischer Effekte im Rahmen einer Neugestaltung der Erhebung sowie insbesondere aufgrund der Folgen der Corona-Pandemie in Ihrer Datenqualität eingeschränkt. Auf die Verwendung dieser Ergebnisse wird daher verzichtet. Weitere Informationen zur methodischen Neugestaltung des Mikrozensus ab 2020 und zu den Auswirkungen der Neugestaltung und der Corona-Krise auf die Ergebnisse des Jahres 2020 finden Sie auf der Informationsseite des Statistischen Bundesamtes: </t>
-  </si>
-  <si>
     <t>https://www.destatis.de/DE/Themen/Gesellschaft-Umwelt/Bevoelkerung/Haushalte-Familien/Methoden/mikrozensus-2020.html</t>
   </si>
   <si>
@@ -131,19 +122,27 @@
     <t>Migration und Teilhabe in Niedersachsen - Integrationsmonitoring 2026</t>
   </si>
   <si>
-    <t>© Landesamt für Statistik Niedersachsen, Hannover 2026,                                                                          </t>
+    <t>1)  Ab der Veröffentlichung der Endergebnisse 2023 und der Erstergebnisse 2024 werden für die Hochrechnung des Mikrozensus Daten der Bevölkerungsfortschreibung herangezogen, die auf den Eckwerten des Zensus 2022 basieren. Die Hochrechnung für die Jahre vor 2011 sowie für bislang veröffentlichte Ergebnisse des Mikrozensus 2011-2013 basiert auf den fortgeschriebenen Ergebnissen der Volkszählung 1987. In 2016 erfolgte die Umstellung auf eine neue Mikrozensus-Stichprobe (auf Basis des Zensus 2011). Ab 2017 wird nur noch die Bevölkerung in Privathaushalten (ohne Gemeinschaftsunterkünfte) ausgewiesen. Dadurch ergibt sich jeweils eine eingeschränkte Vergleichbarkeit mit den Vorjahren.</t>
+  </si>
+  <si>
+    <t>2) Seit dem Jahr 2018 wird im Mikrozensus der Migrationshintergrund im weiteren Sinne jährlich berichtet. Die in der Tabelle ab dem Jahr 2018 abgebildeten Daten zum Migrationshintergrund entsprechen dem Migrationshintergrund im weiteren Sinne, bis 2017 wird der Migrationshintergrund im engeren Sinne abgebildet. Die Vergleichbarkeit ist dadurch eingeschränkt.</t>
+  </si>
+  <si>
+    <t>3) Die Ergebnisse des Mikrozensus 2020 sind unter anderem aufgrund methodischer Effekte im Rahmen einer Neugestaltung der Erhebung sowie insbesondere aufgrund der Folgen der Corona-Pandemie in Ihrer Datenqualität eingeschränkt. Auf die Verwendung dieser Ergebnisse wird daher verzichtet. Weitere Informationen zur methodischen Neugestaltung des Mikrozensus ab 2020 und zu den Auswirkungen der Neugestaltung und der Corona-Krise auf die Ergebnisse des Jahres 2020 finden Sie auf der Informationsseite des Statistischen Bundesamtes:</t>
+  </si>
+  <si>
+    <t>© Landesamt für Statistik Niedersachsen, Hannover 2026,</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="3">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="#\ ##0.0"/>
     <numFmt numFmtId="165" formatCode="#,##0.0"/>
-    <numFmt numFmtId="166" formatCode="0.0"/>
   </numFmts>
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -193,10 +192,6 @@
       <sz val="6"/>
       <color theme="10"/>
       <name val="NDSFrutiger 45 Light"/>
-    </font>
-    <font>
-      <sz val="6"/>
-      <name val="NDSFrutiger 55 Roman"/>
     </font>
   </fonts>
   <fills count="2">
@@ -297,7 +292,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="2"/>
@@ -320,26 +315,12 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="3" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="3"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="3" applyFont="1"/>
-    <xf numFmtId="166" fontId="9" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -349,12 +330,6 @@
     </xf>
     <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -371,6 +346,20 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Link" xfId="1" builtinId="8"/>
@@ -392,9 +381,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 – 2022-Design">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 – 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -432,7 +421,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 – 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -538,7 +527,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 – 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -680,7 +669,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -688,6 +677,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{75ADC1A0-2E9E-4486-AEF7-FD006F785543}">
+  <sheetPr codeName="Tabelle1"/>
   <dimension ref="A1:M85"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -697,7 +687,7 @@
   <sheetData>
     <row r="1" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B1" s="1" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="C1" s="2"/>
       <c r="D1" s="2"/>
@@ -742,25 +732,25 @@
       <c r="I4" s="4"/>
     </row>
     <row r="6" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="23" t="s">
+      <c r="B6" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="C6" s="23" t="s">
+      <c r="C6" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="D6" s="26" t="s">
+      <c r="D6" s="18" t="s">
         <v>4</v>
       </c>
-      <c r="E6" s="27"/>
-      <c r="F6" s="27"/>
-      <c r="G6" s="27"/>
-      <c r="H6" s="27"/>
-      <c r="I6" s="27"/>
-      <c r="J6" s="27"/>
+      <c r="E6" s="19"/>
+      <c r="F6" s="19"/>
+      <c r="G6" s="19"/>
+      <c r="H6" s="19"/>
+      <c r="I6" s="19"/>
+      <c r="J6" s="19"/>
     </row>
     <row r="7" spans="2:10" ht="41.25" x14ac:dyDescent="0.25">
-      <c r="B7" s="24"/>
-      <c r="C7" s="24"/>
+      <c r="B7" s="16"/>
+      <c r="C7" s="16"/>
       <c r="D7" s="5" t="s">
         <v>5</v>
       </c>
@@ -784,908 +774,908 @@
       </c>
     </row>
     <row r="8" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B8" s="25"/>
-      <c r="C8" s="25"/>
-      <c r="D8" s="26" t="s">
+      <c r="B8" s="17"/>
+      <c r="C8" s="17"/>
+      <c r="D8" s="18" t="s">
         <v>12</v>
       </c>
-      <c r="E8" s="27"/>
-      <c r="F8" s="27"/>
-      <c r="G8" s="27"/>
-      <c r="H8" s="27"/>
-      <c r="I8" s="27"/>
-      <c r="J8" s="27"/>
+      <c r="E8" s="19"/>
+      <c r="F8" s="19"/>
+      <c r="G8" s="19"/>
+      <c r="H8" s="19"/>
+      <c r="I8" s="19"/>
+      <c r="J8" s="19"/>
     </row>
     <row r="9" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="18" t="s">
-        <v>13</v>
-      </c>
-      <c r="C9" s="18">
+      <c r="B9" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="C9" s="12">
         <v>2025</v>
       </c>
-      <c r="D9" s="19">
+      <c r="D9" s="13">
         <v>5784.797157</v>
       </c>
-      <c r="E9" s="19">
+      <c r="E9" s="13">
         <v>2646.5485319999998</v>
       </c>
-      <c r="F9" s="19">
+      <c r="F9" s="13">
         <v>168.91743099999999</v>
       </c>
-      <c r="G9" s="19">
+      <c r="G9" s="13">
         <v>1573.325758</v>
       </c>
-      <c r="H9" s="19">
+      <c r="H9" s="13">
         <v>1142.722673</v>
       </c>
-      <c r="I9" s="19">
+      <c r="I9" s="13">
         <v>55.312877999999998</v>
       </c>
-      <c r="J9" s="19">
+      <c r="J9" s="13">
         <v>197.969885</v>
       </c>
     </row>
     <row r="10" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="C10" s="18">
+      <c r="B10" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C10" s="12">
         <v>2025</v>
       </c>
-      <c r="D10" s="19">
+      <c r="D10" s="13">
         <v>2127.741853</v>
       </c>
-      <c r="E10" s="19">
+      <c r="E10" s="13">
         <v>895.07401300000004</v>
       </c>
-      <c r="F10" s="19">
+      <c r="F10" s="13">
         <v>247.47972300000001</v>
       </c>
-      <c r="G10" s="19">
+      <c r="G10" s="13">
         <v>204.98495</v>
       </c>
-      <c r="H10" s="19">
+      <c r="H10" s="13">
         <v>611.61364300000002</v>
       </c>
-      <c r="I10" s="19">
+      <c r="I10" s="13">
         <v>55.849573999999997</v>
       </c>
-      <c r="J10" s="19">
+      <c r="J10" s="13">
         <v>112.73994999999999</v>
       </c>
     </row>
     <row r="11" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="18" t="s">
-        <v>13</v>
-      </c>
-      <c r="C11" s="18">
+      <c r="B11" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="C11" s="12">
         <v>2024</v>
       </c>
-      <c r="D11" s="19">
+      <c r="D11" s="13">
         <v>5812.2569389999999</v>
       </c>
-      <c r="E11" s="19">
+      <c r="E11" s="13">
         <v>2667.337149</v>
       </c>
-      <c r="F11" s="19">
+      <c r="F11" s="13">
         <v>155.398888</v>
       </c>
-      <c r="G11" s="19">
+      <c r="G11" s="13">
         <v>1568.245365</v>
       </c>
-      <c r="H11" s="19">
+      <c r="H11" s="13">
         <v>1168.5717070000001</v>
       </c>
-      <c r="I11" s="19">
+      <c r="I11" s="13">
         <v>58.119768999999998</v>
       </c>
-      <c r="J11" s="19">
+      <c r="J11" s="13">
         <v>194.58406099999996</v>
       </c>
     </row>
     <row r="12" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B12" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="C12" s="18">
+      <c r="B12" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C12" s="12">
         <v>2024</v>
       </c>
-      <c r="D12" s="19">
+      <c r="D12" s="13">
         <v>2108.566898</v>
       </c>
-      <c r="E12" s="19">
+      <c r="E12" s="13">
         <v>875.358428</v>
       </c>
-      <c r="F12" s="19">
+      <c r="F12" s="13">
         <v>247.13717600000001</v>
       </c>
-      <c r="G12" s="19">
+      <c r="G12" s="13">
         <v>210.193262</v>
       </c>
-      <c r="H12" s="19">
+      <c r="H12" s="13">
         <v>602.84329100000002</v>
       </c>
-      <c r="I12" s="19">
+      <c r="I12" s="13">
         <v>61.026826999999997</v>
       </c>
-      <c r="J12" s="19">
+      <c r="J12" s="13">
         <v>112.007914</v>
       </c>
     </row>
     <row r="13" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B13" s="18" t="s">
-        <v>13</v>
-      </c>
-      <c r="C13" s="18">
+      <c r="B13" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="C13" s="12">
         <v>2023</v>
       </c>
-      <c r="D13" s="19">
+      <c r="D13" s="13">
         <v>5927.2500280000013</v>
       </c>
-      <c r="E13" s="19">
+      <c r="E13" s="13">
         <v>2737.2947330000002</v>
       </c>
-      <c r="F13" s="19">
+      <c r="F13" s="13">
         <v>159.35100299999999</v>
       </c>
-      <c r="G13" s="19">
+      <c r="G13" s="13">
         <v>1567.4829970000001</v>
       </c>
-      <c r="H13" s="19">
+      <c r="H13" s="13">
         <v>1212.2092700000001</v>
       </c>
-      <c r="I13" s="19">
+      <c r="I13" s="13">
         <v>57.388255999999998</v>
       </c>
-      <c r="J13" s="19">
+      <c r="J13" s="13">
         <v>193.52376899999999</v>
       </c>
     </row>
     <row r="14" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="C14" s="18">
+      <c r="B14" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C14" s="12">
         <v>2023</v>
       </c>
-      <c r="D14" s="19">
+      <c r="D14" s="13">
         <v>1977.1603669999997</v>
       </c>
-      <c r="E14" s="19">
+      <c r="E14" s="13">
         <v>808.59620299999995</v>
       </c>
-      <c r="F14" s="19">
+      <c r="F14" s="13">
         <v>248.42204699999999</v>
       </c>
-      <c r="G14" s="19">
+      <c r="G14" s="13">
         <v>190.69550699999999</v>
       </c>
-      <c r="H14" s="19">
+      <c r="H14" s="13">
         <v>585.40226900000005</v>
       </c>
-      <c r="I14" s="19">
+      <c r="I14" s="13">
         <v>47.727291000000001</v>
       </c>
-      <c r="J14" s="19">
+      <c r="J14" s="13">
         <v>96.317050000000009</v>
       </c>
     </row>
     <row r="15" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="18" t="s">
-        <v>13</v>
-      </c>
-      <c r="C15" s="18">
+      <c r="B15" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="C15" s="12">
         <v>2022</v>
       </c>
-      <c r="D15" s="19">
+      <c r="D15" s="13">
         <v>5949.9528930000006</v>
       </c>
-      <c r="E15" s="19">
+      <c r="E15" s="13">
         <v>2712.6327620000002</v>
       </c>
-      <c r="F15" s="19">
+      <c r="F15" s="13">
         <v>156.03676999999999</v>
       </c>
-      <c r="G15" s="19">
+      <c r="G15" s="13">
         <v>1577.6182859999999</v>
       </c>
-      <c r="H15" s="19">
+      <c r="H15" s="13">
         <v>1240.333085</v>
       </c>
-      <c r="I15" s="19">
+      <c r="I15" s="13">
         <v>48.281765999999998</v>
       </c>
-      <c r="J15" s="19">
+      <c r="J15" s="13">
         <v>215.05022400000001</v>
       </c>
     </row>
     <row r="16" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B16" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="C16" s="18">
+      <c r="B16" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C16" s="12">
         <v>2022</v>
       </c>
-      <c r="D16" s="19">
+      <c r="D16" s="13">
         <v>1901.0437259999999</v>
       </c>
-      <c r="E16" s="19">
+      <c r="E16" s="13">
         <v>791.63186599999995</v>
       </c>
-      <c r="F16" s="19">
+      <c r="F16" s="13">
         <v>194.831391</v>
       </c>
-      <c r="G16" s="19">
+      <c r="G16" s="13">
         <v>185.826784</v>
       </c>
-      <c r="H16" s="19">
+      <c r="H16" s="13">
         <v>603.31300699999997</v>
       </c>
-      <c r="I16" s="19">
+      <c r="I16" s="13">
         <v>42.077596999999997</v>
       </c>
-      <c r="J16" s="19">
+      <c r="J16" s="13">
         <v>83.363081000000008</v>
       </c>
     </row>
     <row r="17" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="18" t="s">
-        <v>13</v>
-      </c>
-      <c r="C17" s="18">
+      <c r="B17" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="C17" s="12">
         <v>2021</v>
       </c>
-      <c r="D17" s="19">
+      <c r="D17" s="13">
         <v>5944.9624909999984</v>
       </c>
-      <c r="E17" s="19">
+      <c r="E17" s="13">
         <v>2709.629359</v>
       </c>
-      <c r="F17" s="19">
+      <c r="F17" s="13">
         <v>157.81235699999999</v>
       </c>
-      <c r="G17" s="19">
+      <c r="G17" s="13">
         <v>1558.9248250000001</v>
       </c>
-      <c r="H17" s="19">
+      <c r="H17" s="13">
         <v>1260.374069</v>
       </c>
-      <c r="I17" s="19">
+      <c r="I17" s="13">
         <v>49.197209000000001</v>
       </c>
-      <c r="J17" s="19">
+      <c r="J17" s="13">
         <v>209.02467199999998</v>
       </c>
     </row>
     <row r="18" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="C18" s="18">
+      <c r="B18" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C18" s="12">
         <v>2021</v>
       </c>
-      <c r="D18" s="19">
+      <c r="D18" s="13">
         <v>1806.6768549999999</v>
       </c>
-      <c r="E18" s="19">
+      <c r="E18" s="13">
         <v>739.63828000000001</v>
       </c>
-      <c r="F18" s="19">
+      <c r="F18" s="13">
         <v>164.25168600000001</v>
       </c>
-      <c r="G18" s="19">
+      <c r="G18" s="13">
         <v>190.715597</v>
       </c>
-      <c r="H18" s="19">
+      <c r="H18" s="13">
         <v>596.98005899999998</v>
       </c>
-      <c r="I18" s="19">
+      <c r="I18" s="13">
         <v>33.904470000000003</v>
       </c>
-      <c r="J18" s="19">
+      <c r="J18" s="13">
         <v>81.186762999999999</v>
       </c>
     </row>
     <row r="19" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B19" s="18" t="s">
-        <v>13</v>
-      </c>
-      <c r="C19" s="18">
+      <c r="B19" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="C19" s="12">
         <v>2020</v>
       </c>
-      <c r="D19" s="19">
+      <c r="D19" s="13">
         <v>6097</v>
       </c>
-      <c r="E19" s="19">
+      <c r="E19" s="13">
         <v>2877</v>
       </c>
-      <c r="F19" s="19">
+      <c r="F19" s="13">
         <v>131</v>
       </c>
-      <c r="G19" s="19">
+      <c r="G19" s="13">
         <v>1636</v>
       </c>
-      <c r="H19" s="19">
+      <c r="H19" s="13">
         <v>1205</v>
       </c>
-      <c r="I19" s="19">
+      <c r="I19" s="13">
         <v>39</v>
       </c>
-      <c r="J19" s="19">
+      <c r="J19" s="13">
         <v>209</v>
       </c>
     </row>
     <row r="20" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="C20" s="18">
+      <c r="B20" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C20" s="12">
         <v>2020</v>
       </c>
-      <c r="D20" s="19">
+      <c r="D20" s="13">
         <v>1798</v>
       </c>
-      <c r="E20" s="19">
+      <c r="E20" s="13">
         <v>760</v>
       </c>
-      <c r="F20" s="19">
+      <c r="F20" s="13">
         <v>169</v>
       </c>
-      <c r="G20" s="19">
+      <c r="G20" s="13">
         <v>176</v>
       </c>
-      <c r="H20" s="19">
+      <c r="H20" s="13">
         <v>547</v>
       </c>
-      <c r="I20" s="19">
+      <c r="I20" s="13">
         <v>41</v>
       </c>
-      <c r="J20" s="19">
+      <c r="J20" s="13">
         <v>105</v>
       </c>
     </row>
     <row r="21" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="18" t="s">
-        <v>13</v>
-      </c>
-      <c r="C21" s="18">
+      <c r="B21" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="C21" s="12">
         <v>2019</v>
       </c>
-      <c r="D21" s="19">
+      <c r="D21" s="13">
         <v>6103.5</v>
       </c>
-      <c r="E21" s="19">
+      <c r="E21" s="13">
         <v>2876.7</v>
       </c>
-      <c r="F21" s="19">
+      <c r="F21" s="13">
         <v>150.4</v>
       </c>
-      <c r="G21" s="19">
+      <c r="G21" s="13">
         <v>1534.6</v>
       </c>
-      <c r="H21" s="19">
+      <c r="H21" s="13">
         <v>1362.4</v>
       </c>
-      <c r="I21" s="19">
+      <c r="I21" s="13">
         <v>39</v>
       </c>
-      <c r="J21" s="19">
+      <c r="J21" s="13">
         <v>140.4</v>
       </c>
     </row>
     <row r="22" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B22" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="C22" s="18">
+      <c r="B22" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C22" s="12">
         <v>2019</v>
       </c>
-      <c r="D22" s="19">
+      <c r="D22" s="13">
         <v>1786.4</v>
       </c>
-      <c r="E22" s="19">
+      <c r="E22" s="13">
         <v>727.7</v>
       </c>
-      <c r="F22" s="19">
+      <c r="F22" s="13">
         <v>135.5</v>
       </c>
-      <c r="G22" s="19">
+      <c r="G22" s="13">
         <v>167.3</v>
       </c>
-      <c r="H22" s="19">
+      <c r="H22" s="13">
         <v>625.79999999999995</v>
       </c>
-      <c r="I22" s="19">
+      <c r="I22" s="13">
         <v>40.200000000000003</v>
       </c>
-      <c r="J22" s="19">
+      <c r="J22" s="13">
         <v>89.9</v>
       </c>
     </row>
     <row r="23" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="18" t="s">
-        <v>13</v>
-      </c>
-      <c r="C23" s="18">
+      <c r="B23" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="C23" s="12">
         <v>2018</v>
       </c>
-      <c r="D23" s="19">
+      <c r="D23" s="13">
         <v>6106.2</v>
       </c>
-      <c r="E23" s="19">
+      <c r="E23" s="13">
         <v>2833.6</v>
       </c>
-      <c r="F23" s="19">
+      <c r="F23" s="13">
         <v>155.69999999999999</v>
       </c>
-      <c r="G23" s="19">
+      <c r="G23" s="13">
         <v>1538.7</v>
       </c>
-      <c r="H23" s="19">
+      <c r="H23" s="13">
         <v>1405.5</v>
       </c>
-      <c r="I23" s="19">
+      <c r="I23" s="13">
         <v>31.8</v>
       </c>
-      <c r="J23" s="19">
+      <c r="J23" s="13">
         <v>140.9</v>
       </c>
     </row>
     <row r="24" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B24" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="C24" s="18">
+      <c r="B24" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C24" s="12">
         <v>2018</v>
       </c>
-      <c r="D24" s="19">
+      <c r="D24" s="13">
         <v>1761.3000000000002</v>
       </c>
-      <c r="E24" s="19">
+      <c r="E24" s="13">
         <v>713.1</v>
       </c>
-      <c r="F24" s="19">
+      <c r="F24" s="13">
         <v>134.4</v>
       </c>
-      <c r="G24" s="19">
+      <c r="G24" s="13">
         <v>159.19999999999999</v>
       </c>
-      <c r="H24" s="19">
+      <c r="H24" s="13">
         <v>624.20000000000005</v>
       </c>
-      <c r="I24" s="19">
+      <c r="I24" s="13">
         <v>40.9</v>
       </c>
-      <c r="J24" s="19">
+      <c r="J24" s="13">
         <v>89.5</v>
       </c>
     </row>
     <row r="25" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="18" t="s">
-        <v>13</v>
-      </c>
-      <c r="C25" s="18">
+      <c r="B25" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="C25" s="12">
         <v>2017</v>
       </c>
-      <c r="D25" s="19">
+      <c r="D25" s="13">
         <v>6227</v>
       </c>
-      <c r="E25" s="19">
+      <c r="E25" s="13">
         <v>2869</v>
       </c>
-      <c r="F25" s="19">
+      <c r="F25" s="13">
         <v>164</v>
       </c>
-      <c r="G25" s="19">
+      <c r="G25" s="13">
         <v>1515</v>
       </c>
-      <c r="H25" s="19">
+      <c r="H25" s="13">
         <v>1451</v>
       </c>
-      <c r="I25" s="19">
+      <c r="I25" s="13">
         <v>43</v>
       </c>
-      <c r="J25" s="19">
+      <c r="J25" s="13">
         <v>185</v>
       </c>
     </row>
     <row r="26" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B26" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="C26" s="18">
+      <c r="B26" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C26" s="12">
         <v>2017</v>
       </c>
-      <c r="D26" s="19">
+      <c r="D26" s="13">
         <v>1701</v>
       </c>
-      <c r="E26" s="19">
+      <c r="E26" s="13">
         <v>642</v>
       </c>
-      <c r="F26" s="19">
+      <c r="F26" s="13">
         <v>123</v>
       </c>
-      <c r="G26" s="19">
+      <c r="G26" s="13">
         <v>160</v>
       </c>
-      <c r="H26" s="19">
+      <c r="H26" s="13">
         <v>612</v>
       </c>
-      <c r="I26" s="19">
+      <c r="I26" s="13">
         <v>46</v>
       </c>
-      <c r="J26" s="19">
+      <c r="J26" s="13">
         <v>118</v>
       </c>
     </row>
     <row r="27" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B27" s="18" t="s">
-        <v>13</v>
-      </c>
-      <c r="C27" s="18">
+      <c r="B27" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="C27" s="12">
         <v>2016</v>
       </c>
-      <c r="D27" s="19">
+      <c r="D27" s="13">
         <v>6399</v>
       </c>
-      <c r="E27" s="19">
+      <c r="E27" s="13">
         <v>2881</v>
       </c>
-      <c r="F27" s="19">
+      <c r="F27" s="13">
         <v>178</v>
       </c>
-      <c r="G27" s="19">
+      <c r="G27" s="13">
         <v>1593</v>
       </c>
-      <c r="H27" s="19">
+      <c r="H27" s="13">
         <v>1547</v>
       </c>
-      <c r="I27" s="19">
+      <c r="I27" s="13">
         <v>62</v>
       </c>
-      <c r="J27" s="19">
+      <c r="J27" s="13">
         <v>138</v>
       </c>
     </row>
     <row r="28" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B28" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="C28" s="18">
+      <c r="B28" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C28" s="12">
         <v>2016</v>
       </c>
-      <c r="D28" s="19">
+      <c r="D28" s="13">
         <v>1594</v>
       </c>
-      <c r="E28" s="19">
+      <c r="E28" s="13">
         <v>594</v>
       </c>
-      <c r="F28" s="19">
+      <c r="F28" s="13">
         <v>108</v>
       </c>
-      <c r="G28" s="19">
+      <c r="G28" s="13">
         <v>152</v>
       </c>
-      <c r="H28" s="19">
+      <c r="H28" s="13">
         <v>585</v>
       </c>
-      <c r="I28" s="19">
+      <c r="I28" s="13">
         <v>55</v>
       </c>
-      <c r="J28" s="19">
+      <c r="J28" s="13">
         <v>100</v>
       </c>
     </row>
     <row r="29" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B29" s="18" t="s">
-        <v>13</v>
-      </c>
-      <c r="C29" s="18">
+      <c r="B29" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="C29" s="12">
         <v>2015</v>
       </c>
-      <c r="D29" s="19">
+      <c r="D29" s="13">
         <v>6457</v>
       </c>
-      <c r="E29" s="19">
+      <c r="E29" s="13">
         <v>2863</v>
       </c>
-      <c r="F29" s="19">
+      <c r="F29" s="13">
         <v>202</v>
       </c>
-      <c r="G29" s="19">
+      <c r="G29" s="13">
         <v>1608</v>
       </c>
-      <c r="H29" s="19">
+      <c r="H29" s="13">
         <v>1591</v>
       </c>
-      <c r="I29" s="19">
+      <c r="I29" s="13">
         <v>54</v>
       </c>
-      <c r="J29" s="19">
+      <c r="J29" s="13">
         <v>139</v>
       </c>
     </row>
     <row r="30" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B30" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="C30" s="18">
+      <c r="B30" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C30" s="12">
         <v>2015</v>
       </c>
-      <c r="D30" s="19">
+      <c r="D30" s="13">
         <v>1408</v>
       </c>
-      <c r="E30" s="19">
+      <c r="E30" s="13">
         <v>532</v>
       </c>
-      <c r="F30" s="19">
+      <c r="F30" s="13">
         <v>112</v>
       </c>
-      <c r="G30" s="19">
+      <c r="G30" s="13">
         <v>143</v>
       </c>
-      <c r="H30" s="19">
+      <c r="H30" s="13">
         <v>540</v>
       </c>
-      <c r="I30" s="19">
+      <c r="I30" s="13">
         <v>40</v>
       </c>
-      <c r="J30" s="19">
+      <c r="J30" s="13">
         <v>41</v>
       </c>
     </row>
     <row r="31" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B31" s="18" t="s">
-        <v>13</v>
-      </c>
-      <c r="C31" s="18">
+      <c r="B31" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="C31" s="12">
         <v>2014</v>
       </c>
-      <c r="D31" s="19">
+      <c r="D31" s="13">
         <v>6429</v>
       </c>
-      <c r="E31" s="19">
+      <c r="E31" s="13">
         <v>2820</v>
       </c>
-      <c r="F31" s="19">
+      <c r="F31" s="13">
         <v>211</v>
       </c>
-      <c r="G31" s="19">
+      <c r="G31" s="13">
         <v>1575</v>
       </c>
-      <c r="H31" s="19">
+      <c r="H31" s="13">
         <v>1657</v>
       </c>
-      <c r="I31" s="19">
+      <c r="I31" s="13">
         <v>62</v>
       </c>
-      <c r="J31" s="19">
+      <c r="J31" s="13">
         <v>104</v>
       </c>
     </row>
     <row r="32" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B32" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="C32" s="18">
+      <c r="B32" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C32" s="12">
         <v>2014</v>
       </c>
-      <c r="D32" s="19">
+      <c r="D32" s="13">
         <v>1362</v>
       </c>
-      <c r="E32" s="19">
+      <c r="E32" s="13">
         <v>520</v>
       </c>
-      <c r="F32" s="19">
+      <c r="F32" s="13">
         <v>99</v>
       </c>
-      <c r="G32" s="19">
+      <c r="G32" s="13">
         <v>140</v>
       </c>
-      <c r="H32" s="19">
+      <c r="H32" s="13">
         <v>547</v>
       </c>
-      <c r="I32" s="19">
+      <c r="I32" s="13">
         <v>30</v>
       </c>
-      <c r="J32" s="19">
+      <c r="J32" s="13">
         <v>26</v>
       </c>
     </row>
     <row r="33" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B33" s="18" t="s">
-        <v>13</v>
-      </c>
-      <c r="C33" s="18">
+      <c r="B33" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="C33" s="12">
         <v>2013</v>
       </c>
-      <c r="D33" s="19">
+      <c r="D33" s="13">
         <v>6373</v>
       </c>
-      <c r="E33" s="19">
+      <c r="E33" s="13">
         <v>2761</v>
       </c>
-      <c r="F33" s="19">
+      <c r="F33" s="13">
         <v>211</v>
       </c>
-      <c r="G33" s="19">
+      <c r="G33" s="13">
         <v>1581</v>
       </c>
-      <c r="H33" s="19">
+      <c r="H33" s="13">
         <v>1683</v>
       </c>
-      <c r="I33" s="19">
+      <c r="I33" s="13">
         <v>45</v>
       </c>
-      <c r="J33" s="19">
+      <c r="J33" s="13">
         <v>92</v>
       </c>
     </row>
     <row r="34" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B34" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="C34" s="18">
+      <c r="B34" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C34" s="12">
         <v>2013</v>
       </c>
-      <c r="D34" s="19">
+      <c r="D34" s="13">
         <v>1409</v>
       </c>
-      <c r="E34" s="19">
+      <c r="E34" s="13">
         <v>550</v>
       </c>
-      <c r="F34" s="19">
+      <c r="F34" s="13">
         <v>110</v>
       </c>
-      <c r="G34" s="19">
+      <c r="G34" s="13">
         <v>137</v>
       </c>
-      <c r="H34" s="19">
+      <c r="H34" s="13">
         <v>557</v>
       </c>
-      <c r="I34" s="19">
+      <c r="I34" s="13">
         <v>25</v>
       </c>
-      <c r="J34" s="19">
+      <c r="J34" s="13">
         <v>30</v>
       </c>
     </row>
     <row r="35" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B35" s="18" t="s">
-        <v>13</v>
-      </c>
-      <c r="C35" s="18">
+      <c r="B35" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="C35" s="12">
         <v>2012</v>
       </c>
-      <c r="D35" s="19">
+      <c r="D35" s="13">
         <v>6490</v>
       </c>
-      <c r="E35" s="19">
+      <c r="E35" s="13">
         <v>2787</v>
       </c>
-      <c r="F35" s="19">
+      <c r="F35" s="13">
         <v>214</v>
       </c>
-      <c r="G35" s="19">
+      <c r="G35" s="13">
         <v>1577</v>
       </c>
-      <c r="H35" s="19">
+      <c r="H35" s="13">
         <v>1727</v>
       </c>
-      <c r="I35" s="19">
+      <c r="I35" s="13">
         <v>49</v>
       </c>
-      <c r="J35" s="19">
+      <c r="J35" s="13">
         <v>136</v>
       </c>
     </row>
     <row r="36" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B36" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="C36" s="18">
+      <c r="B36" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C36" s="12">
         <v>2012</v>
       </c>
-      <c r="D36" s="19">
+      <c r="D36" s="13">
         <v>1311</v>
       </c>
-      <c r="E36" s="19">
+      <c r="E36" s="13">
         <v>488</v>
       </c>
-      <c r="F36" s="19">
+      <c r="F36" s="13">
         <v>103</v>
       </c>
-      <c r="G36" s="19">
+      <c r="G36" s="13">
         <v>131</v>
       </c>
-      <c r="H36" s="19">
+      <c r="H36" s="13">
         <v>528</v>
       </c>
-      <c r="I36" s="19">
+      <c r="I36" s="13">
         <v>25</v>
       </c>
-      <c r="J36" s="19">
+      <c r="J36" s="13">
         <v>36</v>
       </c>
     </row>
     <row r="37" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B37" s="18" t="s">
-        <v>13</v>
-      </c>
-      <c r="C37" s="18">
+      <c r="B37" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="C37" s="12">
         <v>2011</v>
       </c>
-      <c r="D37" s="19">
+      <c r="D37" s="13">
         <v>6517</v>
       </c>
-      <c r="E37" s="19">
+      <c r="E37" s="13">
         <v>2794</v>
       </c>
-      <c r="F37" s="19">
+      <c r="F37" s="13">
         <v>232</v>
       </c>
-      <c r="G37" s="19">
+      <c r="G37" s="13">
         <v>1593</v>
       </c>
-      <c r="H37" s="19">
+      <c r="H37" s="13">
         <v>1714</v>
       </c>
-      <c r="I37" s="19">
+      <c r="I37" s="13">
         <v>51</v>
       </c>
-      <c r="J37" s="19">
+      <c r="J37" s="13">
         <v>133</v>
       </c>
     </row>
     <row r="38" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B38" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="C38" s="18">
+      <c r="B38" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C38" s="12">
         <v>2011</v>
       </c>
-      <c r="D38" s="19">
+      <c r="D38" s="13">
         <v>1273</v>
       </c>
-      <c r="E38" s="19">
+      <c r="E38" s="13">
         <v>473</v>
       </c>
-      <c r="F38" s="19">
+      <c r="F38" s="13">
         <v>112</v>
       </c>
-      <c r="G38" s="19">
+      <c r="G38" s="13">
         <v>126</v>
       </c>
-      <c r="H38" s="19">
+      <c r="H38" s="13">
         <v>504</v>
       </c>
-      <c r="I38" s="19">
+      <c r="I38" s="13">
         <v>28</v>
       </c>
-      <c r="J38" s="19">
+      <c r="J38" s="13">
         <v>30</v>
       </c>
     </row>
     <row r="41" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B41" s="23" t="s">
+      <c r="B41" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="C41" s="23" t="s">
+      <c r="C41" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="D41" s="26" t="s">
+      <c r="D41" s="18" t="s">
         <v>4</v>
       </c>
-      <c r="E41" s="27"/>
-      <c r="F41" s="27"/>
-      <c r="G41" s="27"/>
-      <c r="H41" s="27"/>
-      <c r="I41" s="27"/>
-      <c r="J41" s="27"/>
+      <c r="E41" s="19"/>
+      <c r="F41" s="19"/>
+      <c r="G41" s="19"/>
+      <c r="H41" s="19"/>
+      <c r="I41" s="19"/>
+      <c r="J41" s="19"/>
     </row>
     <row r="42" spans="2:10" ht="41.25" x14ac:dyDescent="0.25">
-      <c r="B42" s="24"/>
-      <c r="C42" s="24"/>
+      <c r="B42" s="16"/>
+      <c r="C42" s="16"/>
       <c r="D42" s="5" t="s">
         <v>5</v>
       </c>
@@ -1709,1066 +1699,1097 @@
       </c>
     </row>
     <row r="43" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B43" s="25"/>
-      <c r="C43" s="25"/>
-      <c r="D43" s="26" t="s">
+      <c r="B43" s="17"/>
+      <c r="C43" s="17"/>
+      <c r="D43" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="E43" s="27"/>
-      <c r="F43" s="27"/>
-      <c r="G43" s="27"/>
-      <c r="H43" s="27"/>
-      <c r="I43" s="27"/>
-      <c r="J43" s="27"/>
+      <c r="E43" s="19"/>
+      <c r="F43" s="19"/>
+      <c r="G43" s="19"/>
+      <c r="H43" s="19"/>
+      <c r="I43" s="19"/>
+      <c r="J43" s="19"/>
     </row>
     <row r="44" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B44" s="18" t="s">
-        <v>13</v>
-      </c>
-      <c r="C44" s="18">
+      <c r="B44" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="C44" s="12">
         <v>2025</v>
       </c>
-      <c r="D44" s="20">
+      <c r="D44" s="14">
         <v>99.983831740306698</v>
       </c>
-      <c r="E44" s="20">
+      <c r="E44" s="14">
         <v>45.750066254224578</v>
       </c>
-      <c r="F44" s="20">
+      <c r="F44" s="14">
         <v>2.9200234064490638</v>
       </c>
-      <c r="G44" s="20">
+      <c r="G44" s="14">
         <v>27.197595962309034</v>
       </c>
-      <c r="H44" s="20">
+      <c r="H44" s="14">
         <v>19.753893559037373</v>
       </c>
-      <c r="I44" s="20">
+      <c r="I44" s="14">
         <v>0.95617662121596836</v>
       </c>
-      <c r="J44" s="20">
+      <c r="J44" s="14">
         <v>3.4060759370706823</v>
       </c>
     </row>
     <row r="45" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B45" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="C45" s="18">
+      <c r="B45" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C45" s="12">
         <v>2025</v>
       </c>
-      <c r="D45" s="20">
-        <v>96.641120405685058</v>
-      </c>
-      <c r="E45" s="20">
+      <c r="D45" s="14">
+        <v>99.983831740306698</v>
+      </c>
+      <c r="E45" s="14">
         <v>42.066851847558226</v>
       </c>
-      <c r="F45" s="20">
+      <c r="F45" s="14">
         <v>11.631097195887136</v>
       </c>
-      <c r="G45" s="20">
+      <c r="G45" s="14">
         <v>9.633920097542962</v>
       </c>
-      <c r="H45" s="20">
+      <c r="H45" s="14">
         <v>28.744729636147266</v>
       </c>
-      <c r="I45" s="20">
+      <c r="I45" s="14">
         <v>2.6248284734943361</v>
       </c>
-      <c r="J45" s="20">
-        <v>1.9396931550551328</v>
+      <c r="J45" s="14">
+        <v>5.3</v>
       </c>
     </row>
     <row r="46" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B46" s="18" t="s">
-        <v>13</v>
-      </c>
-      <c r="C46" s="18">
+      <c r="B46" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="C46" s="12">
         <v>2024</v>
       </c>
-      <c r="D46" s="20">
+      <c r="D46" s="14">
         <v>100</v>
       </c>
-      <c r="E46" s="20">
+      <c r="E46" s="14">
         <v>45.891590426814751</v>
       </c>
-      <c r="F46" s="20">
+      <c r="F46" s="14">
         <v>2.6736410594184163</v>
       </c>
-      <c r="G46" s="20">
+      <c r="G46" s="14">
         <v>26.981693711390143</v>
       </c>
-      <c r="H46" s="20">
+      <c r="H46" s="14">
         <v>20.105300217527088</v>
       </c>
-      <c r="I46" s="20">
+      <c r="I46" s="14">
         <v>0.99995181923253929</v>
       </c>
-      <c r="J46" s="20">
+      <c r="J46" s="14">
         <v>3.3478227656170723</v>
       </c>
     </row>
     <row r="47" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B47" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="C47" s="18">
+      <c r="B47" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C47" s="12">
         <v>2024</v>
       </c>
-      <c r="D47" s="20">
+      <c r="D47" s="14">
         <v>100</v>
       </c>
-      <c r="E47" s="20">
+      <c r="E47" s="14">
         <v>41.514377790445614</v>
       </c>
-      <c r="F47" s="20">
+      <c r="F47" s="14">
         <v>11.720622961235541</v>
       </c>
-      <c r="G47" s="20">
+      <c r="G47" s="14">
         <v>9.9685365543474447</v>
       </c>
-      <c r="H47" s="20">
+      <c r="H47" s="14">
         <v>28.590190407134049</v>
       </c>
-      <c r="I47" s="20">
+      <c r="I47" s="14">
         <v>2.8942324314151304</v>
       </c>
-      <c r="J47" s="20">
+      <c r="J47" s="14">
         <v>5.3120398554222206</v>
       </c>
     </row>
     <row r="48" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B48" s="18" t="s">
-        <v>13</v>
-      </c>
-      <c r="C48" s="18">
+      <c r="B48" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="C48" s="12">
         <v>2023</v>
       </c>
-      <c r="D48" s="20">
+      <c r="D48" s="14">
         <v>99.999999999999986</v>
       </c>
-      <c r="E48" s="20">
+      <c r="E48" s="14">
         <v>46.18152971562143</v>
       </c>
-      <c r="F48" s="20">
+      <c r="F48" s="14">
         <v>2.6884474629420838</v>
       </c>
-      <c r="G48" s="20">
+      <c r="G48" s="14">
         <v>26.44536656282926</v>
       </c>
-      <c r="H48" s="20">
+      <c r="H48" s="14">
         <v>20.451461711140755</v>
       </c>
-      <c r="I48" s="20">
+      <c r="I48" s="14">
         <v>0.96821048089588013</v>
       </c>
-      <c r="J48" s="20">
+      <c r="J48" s="14">
         <v>3.2649840665705745</v>
       </c>
     </row>
     <row r="49" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B49" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="C49" s="18">
+      <c r="B49" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C49" s="12">
         <v>2023</v>
       </c>
-      <c r="D49" s="20">
+      <c r="D49" s="14">
         <v>100.00000000000003</v>
       </c>
-      <c r="E49" s="20">
+      <c r="E49" s="14">
         <v>40.896844610885324</v>
       </c>
-      <c r="F49" s="20">
+      <c r="F49" s="14">
         <v>12.564587635192066</v>
       </c>
-      <c r="G49" s="20">
+      <c r="G49" s="14">
         <v>9.6449185499984296</v>
       </c>
-      <c r="H49" s="20">
+      <c r="H49" s="14">
         <v>29.608234049737053</v>
       </c>
-      <c r="I49" s="20">
+      <c r="I49" s="14">
         <v>2.4139312013631926</v>
       </c>
-      <c r="J49" s="20">
+      <c r="J49" s="14">
         <v>4.8714839528239455</v>
       </c>
     </row>
     <row r="50" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B50" s="18" t="s">
-        <v>13</v>
-      </c>
-      <c r="C50" s="18">
+      <c r="B50" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="C50" s="12">
         <v>2022</v>
       </c>
-      <c r="D50" s="20">
+      <c r="D50" s="14">
         <v>99.999999999999972</v>
       </c>
-      <c r="E50" s="20">
+      <c r="E50" s="14">
         <v>45.590827537329879</v>
       </c>
-      <c r="F50" s="20">
+      <c r="F50" s="14">
         <v>2.6224874852971372</v>
       </c>
-      <c r="G50" s="20">
+      <c r="G50" s="14">
         <v>26.514802963499694</v>
       </c>
-      <c r="H50" s="20">
+      <c r="H50" s="14">
         <v>20.846099243226394</v>
       </c>
-      <c r="I50" s="20">
+      <c r="I50" s="14">
         <v>0.81146467658260824</v>
       </c>
-      <c r="J50" s="20">
+      <c r="J50" s="14">
         <v>3.6143180940642781</v>
       </c>
     </row>
     <row r="51" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B51" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="C51" s="18">
+      <c r="B51" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C51" s="12">
         <v>2022</v>
       </c>
-      <c r="D51" s="20">
+      <c r="D51" s="14">
         <v>100</v>
       </c>
-      <c r="E51" s="20">
+      <c r="E51" s="14">
         <v>41.641959896718333</v>
       </c>
-      <c r="F51" s="20">
+      <c r="F51" s="14">
         <v>10.248653849217144</v>
       </c>
-      <c r="G51" s="20">
+      <c r="G51" s="14">
         <v>9.7749873639676625</v>
       </c>
-      <c r="H51" s="20">
+      <c r="H51" s="14">
         <v>31.735882702153063</v>
       </c>
-      <c r="I51" s="20">
+      <c r="I51" s="14">
         <v>2.2133944855932262</v>
       </c>
-      <c r="J51" s="20">
+      <c r="J51" s="14">
         <v>4.3851217023505757</v>
       </c>
     </row>
     <row r="52" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B52" s="18" t="s">
-        <v>13</v>
-      </c>
-      <c r="C52" s="18">
+      <c r="B52" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="C52" s="12">
         <v>2021</v>
       </c>
-      <c r="D52" s="20">
+      <c r="D52" s="14">
         <v>100</v>
       </c>
-      <c r="E52" s="20">
+      <c r="E52" s="14">
         <v>45.578577881728819</v>
       </c>
-      <c r="F52" s="20">
+      <c r="F52" s="14">
         <v>2.6545559747249889</v>
       </c>
-      <c r="G52" s="20">
+      <c r="G52" s="14">
         <v>26.222618348896837</v>
       </c>
-      <c r="H52" s="20">
+      <c r="H52" s="14">
         <v>21.200706832180423</v>
       </c>
-      <c r="I52" s="20">
+      <c r="I52" s="14">
         <v>0.82754448113808976</v>
       </c>
-      <c r="J52" s="20">
+      <c r="J52" s="14">
         <v>3.5159964813308702</v>
       </c>
     </row>
     <row r="53" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B53" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="C53" s="18">
+      <c r="B53" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C53" s="12">
         <v>2021</v>
       </c>
-      <c r="D53" s="20">
+      <c r="D53" s="14">
         <v>100</v>
       </c>
-      <c r="E53" s="20">
+      <c r="E53" s="14">
         <v>40.939157323737348</v>
       </c>
-      <c r="F53" s="20">
+      <c r="F53" s="14">
         <v>9.091370465361944</v>
       </c>
-      <c r="G53" s="20">
+      <c r="G53" s="14">
         <v>10.556154326779152</v>
       </c>
-      <c r="H53" s="20">
+      <c r="H53" s="14">
         <v>33.042990358118033</v>
       </c>
-      <c r="I53" s="20">
+      <c r="I53" s="14">
         <v>1.8766205979873476</v>
       </c>
-      <c r="J53" s="20">
+      <c r="J53" s="14">
         <v>4.4937069280161888</v>
       </c>
     </row>
     <row r="54" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B54" s="18" t="s">
-        <v>13</v>
-      </c>
-      <c r="C54" s="18">
+      <c r="B54" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="C54" s="12">
         <v>2020</v>
       </c>
-      <c r="D54" s="20">
+      <c r="D54" s="14">
         <v>99.999999999999986</v>
       </c>
-      <c r="E54" s="20">
+      <c r="E54" s="14">
         <v>47.187141216991961</v>
       </c>
-      <c r="F54" s="20">
+      <c r="F54" s="14">
         <v>2.1485976709857306</v>
       </c>
-      <c r="G54" s="20">
+      <c r="G54" s="14">
         <v>26.832868623913399</v>
       </c>
-      <c r="H54" s="20">
+      <c r="H54" s="14">
         <v>19.763818271280957</v>
       </c>
-      <c r="I54" s="20">
+      <c r="I54" s="14">
         <v>0.63965884861407252</v>
       </c>
-      <c r="J54" s="20">
+      <c r="J54" s="14">
         <v>3.4279153682138754</v>
       </c>
     </row>
     <row r="55" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B55" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="C55" s="18">
+      <c r="B55" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C55" s="12">
         <v>2020</v>
       </c>
-      <c r="D55" s="20">
+      <c r="D55" s="14">
         <v>100</v>
       </c>
-      <c r="E55" s="20">
+      <c r="E55" s="14">
         <v>42.269187986651836</v>
       </c>
-      <c r="F55" s="20">
+      <c r="F55" s="14">
         <v>9.3993325917686317</v>
       </c>
-      <c r="G55" s="20">
+      <c r="G55" s="14">
         <v>9.788654060066742</v>
       </c>
-      <c r="H55" s="20">
+      <c r="H55" s="14">
         <v>30.42269187986652</v>
       </c>
-      <c r="I55" s="20">
+      <c r="I55" s="14">
         <v>2.2803114571746388</v>
       </c>
-      <c r="J55" s="20">
+      <c r="J55" s="14">
         <v>5.8398220244716352</v>
       </c>
     </row>
     <row r="56" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B56" s="18" t="s">
-        <v>13</v>
-      </c>
-      <c r="C56" s="18">
+      <c r="B56" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="C56" s="12">
         <v>2019</v>
       </c>
-      <c r="D56" s="20">
+      <c r="D56" s="14">
         <v>100</v>
       </c>
-      <c r="E56" s="20">
+      <c r="E56" s="14">
         <v>47.131973457852048</v>
       </c>
-      <c r="F56" s="20">
+      <c r="F56" s="14">
         <v>2.464159908249365</v>
       </c>
-      <c r="G56" s="20">
+      <c r="G56" s="14">
         <v>25.142950765953959</v>
       </c>
-      <c r="H56" s="20">
+      <c r="H56" s="14">
         <v>22.321618743343986</v>
       </c>
-      <c r="I56" s="20">
+      <c r="I56" s="14">
         <v>0.63897763578274758</v>
       </c>
-      <c r="J56" s="20">
+      <c r="J56" s="14">
         <v>2.3003194888178915</v>
       </c>
     </row>
     <row r="57" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B57" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="C57" s="18">
+      <c r="B57" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C57" s="12">
         <v>2019</v>
       </c>
-      <c r="D57" s="20">
+      <c r="D57" s="14">
         <v>100</v>
       </c>
-      <c r="E57" s="20">
+      <c r="E57" s="14">
         <v>40.735557545902374</v>
       </c>
-      <c r="F57" s="20">
+      <c r="F57" s="14">
         <v>7.5850873264666356</v>
       </c>
-      <c r="G57" s="20">
+      <c r="G57" s="14">
         <v>9.3652037617554864</v>
       </c>
-      <c r="H57" s="20">
+      <c r="H57" s="14">
         <v>35.031347962382441</v>
       </c>
-      <c r="I57" s="20">
+      <c r="I57" s="14">
         <v>2.2503358710255261</v>
       </c>
-      <c r="J57" s="20">
+      <c r="J57" s="14">
         <v>5.0324675324675328</v>
       </c>
     </row>
     <row r="58" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B58" s="18" t="s">
-        <v>13</v>
-      </c>
-      <c r="C58" s="18">
+      <c r="B58" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="C58" s="12">
         <v>2018</v>
       </c>
-      <c r="D58" s="20">
+      <c r="D58" s="14">
         <v>100.00000000000001</v>
       </c>
-      <c r="E58" s="20">
+      <c r="E58" s="14">
         <v>46.405292980904655</v>
       </c>
-      <c r="F58" s="20">
+      <c r="F58" s="14">
         <v>2.5498673479414364</v>
       </c>
-      <c r="G58" s="20">
+      <c r="G58" s="14">
         <v>25.198978087845141</v>
       </c>
-      <c r="H58" s="20">
+      <c r="H58" s="14">
         <v>23.017588680357669</v>
       </c>
-      <c r="I58" s="20">
+      <c r="I58" s="14">
         <v>0.52078215584160359</v>
       </c>
-      <c r="J58" s="20">
+      <c r="J58" s="14">
         <v>2.3074907471094952</v>
       </c>
     </row>
     <row r="59" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B59" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="C59" s="18">
+      <c r="B59" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C59" s="12">
         <v>2018</v>
       </c>
-      <c r="D59" s="20">
+      <c r="D59" s="14">
         <v>100</v>
       </c>
-      <c r="E59" s="20">
+      <c r="E59" s="14">
         <v>40.487140180548451</v>
       </c>
-      <c r="F59" s="20">
+      <c r="F59" s="14">
         <v>7.6307273036961334</v>
       </c>
-      <c r="G59" s="20">
+      <c r="G59" s="14">
         <v>9.0387781752114904</v>
       </c>
-      <c r="H59" s="20">
+      <c r="H59" s="14">
         <v>35.439732016124452</v>
       </c>
-      <c r="I59" s="20">
+      <c r="I59" s="14">
         <v>2.3221484131039567</v>
       </c>
-      <c r="J59" s="20">
+      <c r="J59" s="14">
         <v>5.0814739113155056</v>
       </c>
     </row>
     <row r="60" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B60" s="18" t="s">
-        <v>13</v>
-      </c>
-      <c r="C60" s="18">
+      <c r="B60" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="C60" s="12">
         <v>2017</v>
       </c>
-      <c r="D60" s="20">
+      <c r="D60" s="14">
         <v>100</v>
       </c>
-      <c r="E60" s="20">
+      <c r="E60" s="14">
         <v>46.073550666452547</v>
       </c>
-      <c r="F60" s="20">
+      <c r="F60" s="14">
         <v>2.6336919865103581</v>
       </c>
-      <c r="G60" s="20">
+      <c r="G60" s="14">
         <v>24.32953268026337</v>
       </c>
-      <c r="H60" s="20">
+      <c r="H60" s="14">
         <v>23.301750441625181</v>
       </c>
-      <c r="I60" s="20">
+      <c r="I60" s="14">
         <v>0.69054119158503291</v>
       </c>
-      <c r="J60" s="20">
+      <c r="J60" s="14">
         <v>2.9709330335635138</v>
       </c>
     </row>
     <row r="61" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B61" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="C61" s="18">
+      <c r="B61" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C61" s="12">
         <v>2017</v>
       </c>
-      <c r="D61" s="20">
+      <c r="D61" s="14">
         <v>100</v>
       </c>
-      <c r="E61" s="20">
+      <c r="E61" s="14">
         <v>37.742504409171076</v>
       </c>
-      <c r="F61" s="20">
+      <c r="F61" s="14">
         <v>7.2310405643738971</v>
       </c>
-      <c r="G61" s="20">
+      <c r="G61" s="14">
         <v>9.4062316284538507</v>
       </c>
-      <c r="H61" s="20">
+      <c r="H61" s="14">
         <v>35.978835978835974</v>
       </c>
-      <c r="I61" s="20">
+      <c r="I61" s="14">
         <v>2.7042915931804821</v>
       </c>
-      <c r="J61" s="20">
+      <c r="J61" s="14">
         <v>6.9370958259847155</v>
       </c>
     </row>
     <row r="62" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B62" s="18" t="s">
-        <v>13</v>
-      </c>
-      <c r="C62" s="18">
+      <c r="B62" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="C62" s="12">
         <v>2016</v>
       </c>
-      <c r="D62" s="20">
+      <c r="D62" s="14">
         <v>100</v>
       </c>
-      <c r="E62" s="20">
+      <c r="E62" s="14">
         <v>45.022659790592279</v>
       </c>
-      <c r="F62" s="20">
+      <c r="F62" s="14">
         <v>2.7816846382247227</v>
       </c>
-      <c r="G62" s="20">
+      <c r="G62" s="14">
         <v>24.894514767932492</v>
       </c>
-      <c r="H62" s="20">
+      <c r="H62" s="14">
         <v>24.175652445694638</v>
       </c>
-      <c r="I62" s="20">
+      <c r="I62" s="14">
         <v>0.96890139084231908</v>
       </c>
-      <c r="J62" s="20">
+      <c r="J62" s="14">
         <v>2.1565869667135491</v>
       </c>
     </row>
     <row r="63" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B63" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="C63" s="18">
+      <c r="B63" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C63" s="12">
         <v>2016</v>
       </c>
-      <c r="D63" s="20">
+      <c r="D63" s="14">
         <v>100</v>
       </c>
-      <c r="E63" s="20">
+      <c r="E63" s="14">
         <v>37.264742785445421</v>
       </c>
-      <c r="F63" s="20">
+      <c r="F63" s="14">
         <v>6.7754077791718954</v>
       </c>
-      <c r="G63" s="20">
+      <c r="G63" s="14">
         <v>9.5357590966122974</v>
       </c>
-      <c r="H63" s="20">
+      <c r="H63" s="14">
         <v>36.700125470514429</v>
       </c>
-      <c r="I63" s="20">
+      <c r="I63" s="14">
         <v>3.4504391468005018</v>
       </c>
-      <c r="J63" s="20">
+      <c r="J63" s="14">
         <v>6.2735257214554583</v>
       </c>
     </row>
     <row r="64" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B64" s="18" t="s">
-        <v>13</v>
-      </c>
-      <c r="C64" s="18">
+      <c r="B64" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="C64" s="12">
         <v>2015</v>
       </c>
-      <c r="D64" s="20">
+      <c r="D64" s="14">
         <v>100</v>
       </c>
-      <c r="E64" s="20">
+      <c r="E64" s="14">
         <v>44.339476537091528</v>
       </c>
-      <c r="F64" s="20">
+      <c r="F64" s="14">
         <v>3.1283877961901809</v>
       </c>
-      <c r="G64" s="20">
+      <c r="G64" s="14">
         <v>24.903205823137682</v>
       </c>
-      <c r="H64" s="20">
+      <c r="H64" s="14">
         <v>24.639925662072169</v>
       </c>
-      <c r="I64" s="20">
+      <c r="I64" s="14">
         <v>0.83630168809044436</v>
       </c>
-      <c r="J64" s="20">
+      <c r="J64" s="14">
         <v>2.1527024934179959</v>
       </c>
     </row>
     <row r="65" spans="1:13" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B65" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="C65" s="18">
+      <c r="B65" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C65" s="12">
         <v>2015</v>
       </c>
-      <c r="D65" s="20">
+      <c r="D65" s="14">
         <v>100</v>
       </c>
-      <c r="E65" s="20">
+      <c r="E65" s="14">
         <v>37.784090909090914</v>
       </c>
-      <c r="F65" s="20">
+      <c r="F65" s="14">
         <v>7.9545454545454541</v>
       </c>
-      <c r="G65" s="20">
+      <c r="G65" s="14">
         <v>10.15625</v>
       </c>
-      <c r="H65" s="20">
+      <c r="H65" s="14">
         <v>38.352272727272727</v>
       </c>
-      <c r="I65" s="20">
+      <c r="I65" s="14">
         <v>2.8409090909090908</v>
       </c>
-      <c r="J65" s="20">
+      <c r="J65" s="14">
         <v>2.9119318181818179</v>
       </c>
     </row>
     <row r="66" spans="1:13" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B66" s="18" t="s">
-        <v>13</v>
-      </c>
-      <c r="C66" s="18">
+      <c r="B66" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="C66" s="12">
         <v>2014</v>
       </c>
-      <c r="D66" s="20">
+      <c r="D66" s="14">
         <v>100</v>
       </c>
-      <c r="E66" s="20">
+      <c r="E66" s="14">
         <v>43.86374241717219</v>
       </c>
-      <c r="F66" s="20">
+      <c r="F66" s="14">
         <v>3.282003421994089</v>
       </c>
-      <c r="G66" s="20">
+      <c r="G66" s="14">
         <v>24.498366775548298</v>
       </c>
-      <c r="H66" s="20">
+      <c r="H66" s="14">
         <v>25.773837299735575</v>
       </c>
-      <c r="I66" s="20">
+      <c r="I66" s="14">
         <v>0.9643801524342821</v>
       </c>
-      <c r="J66" s="20">
+      <c r="J66" s="14">
         <v>1.6176699331155699</v>
       </c>
     </row>
     <row r="67" spans="1:13" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B67" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="C67" s="18">
+      <c r="B67" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C67" s="12">
         <v>2014</v>
       </c>
-      <c r="D67" s="20">
+      <c r="D67" s="14">
         <v>100.00000000000001</v>
       </c>
-      <c r="E67" s="20">
+      <c r="E67" s="14">
         <v>38.179148311306903</v>
       </c>
-      <c r="F67" s="20">
+      <c r="F67" s="14">
         <v>7.2687224669603516</v>
       </c>
-      <c r="G67" s="20">
+      <c r="G67" s="14">
         <v>10.279001468428781</v>
       </c>
-      <c r="H67" s="20">
+      <c r="H67" s="14">
         <v>40.161527165932455</v>
       </c>
-      <c r="I67" s="20">
+      <c r="I67" s="14">
         <v>2.2026431718061676</v>
       </c>
-      <c r="J67" s="20">
+      <c r="J67" s="14">
         <v>1.908957415565345</v>
       </c>
     </row>
     <row r="68" spans="1:13" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B68" s="18" t="s">
-        <v>13</v>
-      </c>
-      <c r="C68" s="18">
+      <c r="B68" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="C68" s="12">
         <v>2013</v>
       </c>
-      <c r="D68" s="20">
+      <c r="D68" s="14">
         <v>100</v>
       </c>
-      <c r="E68" s="20">
+      <c r="E68" s="14">
         <v>43.32339557508238</v>
       </c>
-      <c r="F68" s="20">
+      <c r="F68" s="14">
         <v>3.3108426172916996</v>
       </c>
-      <c r="G68" s="20">
+      <c r="G68" s="14">
         <v>24.80778283383022</v>
       </c>
-      <c r="H68" s="20">
+      <c r="H68" s="14">
         <v>26.408284952141848</v>
       </c>
-      <c r="I68" s="20">
+      <c r="I68" s="14">
         <v>0.70610387572571787</v>
       </c>
-      <c r="J68" s="20">
+      <c r="J68" s="14">
         <v>1.4435901459281344</v>
       </c>
     </row>
     <row r="69" spans="1:13" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B69" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="C69" s="18">
+      <c r="B69" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C69" s="12">
         <v>2013</v>
       </c>
-      <c r="D69" s="20">
+      <c r="D69" s="14">
         <v>100</v>
       </c>
-      <c r="E69" s="20">
+      <c r="E69" s="14">
         <v>39.034776437189493</v>
       </c>
-      <c r="F69" s="20">
+      <c r="F69" s="14">
         <v>7.8069552874378987</v>
       </c>
-      <c r="G69" s="20">
+      <c r="G69" s="14">
         <v>9.7232079488999279</v>
       </c>
-      <c r="H69" s="20">
+      <c r="H69" s="14">
         <v>39.531582682753722</v>
       </c>
-      <c r="I69" s="20">
+      <c r="I69" s="14">
         <v>1.7743080198722498</v>
       </c>
-      <c r="J69" s="20">
+      <c r="J69" s="14">
         <v>2.1291696238466997</v>
       </c>
     </row>
     <row r="70" spans="1:13" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B70" s="18" t="s">
-        <v>13</v>
-      </c>
-      <c r="C70" s="18">
+      <c r="B70" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="C70" s="12">
         <v>2012</v>
       </c>
-      <c r="D70" s="20">
+      <c r="D70" s="14">
         <v>100</v>
       </c>
-      <c r="E70" s="20">
+      <c r="E70" s="14">
         <v>42.942989214175654</v>
       </c>
-      <c r="F70" s="20">
+      <c r="F70" s="14">
         <v>3.2973805855161791</v>
       </c>
-      <c r="G70" s="20">
+      <c r="G70" s="14">
         <v>24.298921417565484</v>
       </c>
-      <c r="H70" s="20">
+      <c r="H70" s="14">
         <v>26.610169491525426</v>
       </c>
-      <c r="I70" s="20">
+      <c r="I70" s="14">
         <v>0.75500770416024654</v>
       </c>
-      <c r="J70" s="20">
+      <c r="J70" s="14">
         <v>2.0955315870570108</v>
       </c>
     </row>
     <row r="71" spans="1:13" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B71" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="C71" s="18">
+      <c r="B71" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C71" s="12">
         <v>2012</v>
       </c>
-      <c r="D71" s="20">
+      <c r="D71" s="14">
         <v>100</v>
       </c>
-      <c r="E71" s="20">
+      <c r="E71" s="14">
         <v>37.223493516399699</v>
       </c>
-      <c r="F71" s="20">
+      <c r="F71" s="14">
         <v>7.8565980167810832</v>
       </c>
-      <c r="G71" s="20">
+      <c r="G71" s="14">
         <v>9.9923722349351642</v>
       </c>
-      <c r="H71" s="20">
+      <c r="H71" s="14">
         <v>40.274599542334094</v>
       </c>
-      <c r="I71" s="20">
+      <c r="I71" s="14">
         <v>1.9069412662090008</v>
       </c>
-      <c r="J71" s="20">
+      <c r="J71" s="14">
         <v>2.7459954233409611</v>
       </c>
     </row>
     <row r="72" spans="1:13" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B72" s="18" t="s">
-        <v>13</v>
-      </c>
-      <c r="C72" s="18">
+      <c r="B72" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="C72" s="12">
         <v>2011</v>
       </c>
-      <c r="D72" s="20">
+      <c r="D72" s="14">
         <v>100</v>
       </c>
-      <c r="E72" s="20">
+      <c r="E72" s="14">
         <v>42.87248734080098</v>
       </c>
-      <c r="F72" s="20">
+      <c r="F72" s="14">
         <v>3.5599202086849782</v>
       </c>
-      <c r="G72" s="20">
+      <c r="G72" s="14">
         <v>24.443762467392972</v>
       </c>
-      <c r="H72" s="20">
+      <c r="H72" s="14">
         <v>26.300444990026083</v>
       </c>
-      <c r="I72" s="20">
+      <c r="I72" s="14">
         <v>0.78256866656437019</v>
       </c>
-      <c r="J72" s="20">
+      <c r="J72" s="14">
         <v>2.0408163265306123</v>
       </c>
     </row>
     <row r="73" spans="1:13" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B73" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="C73" s="18">
+      <c r="B73" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C73" s="12">
         <v>2011</v>
       </c>
-      <c r="D73" s="20">
+      <c r="D73" s="14">
         <v>100</v>
       </c>
-      <c r="E73" s="20">
+      <c r="E73" s="14">
         <v>37.156323644933231</v>
       </c>
-      <c r="F73" s="20">
+      <c r="F73" s="14">
         <v>8.7981146897093474</v>
       </c>
-      <c r="G73" s="20">
+      <c r="G73" s="14">
         <v>9.8978790259230163</v>
       </c>
-      <c r="H73" s="20">
+      <c r="H73" s="14">
         <v>39.591516103692065</v>
       </c>
-      <c r="I73" s="20">
+      <c r="I73" s="14">
         <v>2.1995286724273369</v>
       </c>
-      <c r="J73" s="20">
+      <c r="J73" s="14">
         <v>2.356637863315004</v>
       </c>
     </row>
     <row r="74" spans="1:13" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A74" s="10"/>
-      <c r="B74" s="13"/>
-      <c r="C74" s="14"/>
-      <c r="D74" s="14"/>
-      <c r="E74" s="14"/>
-      <c r="F74" s="14"/>
-      <c r="G74" s="14"/>
-      <c r="H74" s="14"/>
-      <c r="I74" s="10"/>
-      <c r="J74" s="10"/>
-      <c r="K74" s="10"/>
-      <c r="L74" s="10"/>
-      <c r="M74" s="10"/>
-    </row>
-    <row r="75" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A74" s="9"/>
+      <c r="B74" s="10"/>
+      <c r="C74" s="11"/>
+      <c r="D74" s="11"/>
+      <c r="E74" s="11"/>
+      <c r="F74" s="11"/>
+      <c r="G74" s="11"/>
+      <c r="H74" s="11"/>
+      <c r="I74" s="9"/>
+      <c r="J74" s="9"/>
+      <c r="K74" s="9"/>
+      <c r="L74" s="9"/>
+      <c r="M74" s="9"/>
+    </row>
+    <row r="75" spans="1:13" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A75" s="8"/>
-      <c r="B75" s="21" t="s">
+      <c r="B75" s="20" t="s">
+        <v>22</v>
+      </c>
+      <c r="C75" s="20"/>
+      <c r="D75" s="20"/>
+      <c r="E75" s="20"/>
+      <c r="F75" s="20"/>
+      <c r="G75" s="20"/>
+      <c r="H75" s="20"/>
+      <c r="I75" s="20"/>
+      <c r="J75" s="20"/>
+      <c r="K75" s="20"/>
+      <c r="L75" s="20"/>
+      <c r="M75" s="20"/>
+    </row>
+    <row r="76" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A76" s="9"/>
+      <c r="B76" s="20" t="s">
+        <v>23</v>
+      </c>
+      <c r="C76" s="20"/>
+      <c r="D76" s="20"/>
+      <c r="E76" s="20"/>
+      <c r="F76" s="20"/>
+      <c r="G76" s="20"/>
+      <c r="H76" s="20"/>
+      <c r="I76" s="20"/>
+      <c r="J76" s="20"/>
+      <c r="K76" s="20"/>
+      <c r="L76" s="20"/>
+      <c r="M76" s="20"/>
+    </row>
+    <row r="77" spans="1:13" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A77" s="9"/>
+      <c r="B77" s="20" t="s">
+        <v>24</v>
+      </c>
+      <c r="C77" s="20"/>
+      <c r="D77" s="20"/>
+      <c r="E77" s="20"/>
+      <c r="F77" s="20"/>
+      <c r="G77" s="20"/>
+      <c r="H77" s="20"/>
+      <c r="I77" s="20"/>
+      <c r="J77" s="20"/>
+      <c r="K77" s="20"/>
+      <c r="L77" s="20"/>
+      <c r="M77" s="20"/>
+    </row>
+    <row r="78" spans="1:13" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A78" s="9"/>
+      <c r="B78" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="C75" s="21"/>
-      <c r="D75" s="21"/>
-      <c r="E75" s="21"/>
-      <c r="F75" s="21"/>
-      <c r="G75" s="21"/>
-      <c r="H75" s="21"/>
-      <c r="I75" s="21"/>
-      <c r="J75" s="21"/>
-      <c r="K75" s="9"/>
-      <c r="L75" s="9"/>
-      <c r="M75" s="9"/>
-    </row>
-    <row r="76" spans="1:13" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A76" s="10"/>
-      <c r="B76" s="11" t="s">
+      <c r="C78" s="22"/>
+      <c r="D78" s="22"/>
+      <c r="E78" s="22"/>
+      <c r="F78" s="22"/>
+      <c r="G78" s="22"/>
+      <c r="H78" s="22"/>
+      <c r="I78" s="22"/>
+      <c r="J78" s="22"/>
+      <c r="K78" s="22"/>
+      <c r="L78" s="22"/>
+      <c r="M78" s="22"/>
+    </row>
+    <row r="79" spans="1:13" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A79" s="9"/>
+      <c r="B79" s="21"/>
+      <c r="C79" s="22"/>
+      <c r="D79" s="22"/>
+      <c r="E79" s="22"/>
+      <c r="F79" s="22"/>
+      <c r="G79" s="22"/>
+      <c r="H79" s="22"/>
+      <c r="I79" s="22"/>
+      <c r="J79" s="22"/>
+      <c r="K79" s="22"/>
+      <c r="L79" s="22"/>
+      <c r="M79" s="22"/>
+    </row>
+    <row r="80" spans="1:13" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B80" s="23" t="s">
         <v>17</v>
       </c>
-      <c r="C76" s="10"/>
-      <c r="D76" s="10"/>
-      <c r="E76" s="10"/>
-      <c r="F76" s="10"/>
-      <c r="G76" s="10"/>
-      <c r="H76" s="10"/>
-      <c r="I76" s="10"/>
-      <c r="J76" s="10"/>
-      <c r="K76" s="10"/>
-      <c r="L76" s="10"/>
-      <c r="M76" s="10"/>
-    </row>
-    <row r="77" spans="1:13" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A77" s="10"/>
-      <c r="B77" s="22" t="s">
+      <c r="C80" s="22"/>
+      <c r="D80" s="22"/>
+      <c r="E80" s="22"/>
+      <c r="F80" s="22"/>
+      <c r="G80" s="22"/>
+      <c r="H80" s="22"/>
+      <c r="I80" s="22"/>
+      <c r="J80" s="22"/>
+      <c r="K80" s="22"/>
+      <c r="L80" s="22"/>
+      <c r="M80" s="22"/>
+    </row>
+    <row r="81" spans="2:13" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B81" s="22"/>
+      <c r="C81" s="22"/>
+      <c r="D81" s="22"/>
+      <c r="E81" s="22"/>
+      <c r="F81" s="22"/>
+      <c r="G81" s="22"/>
+      <c r="H81" s="22"/>
+      <c r="I81" s="22"/>
+      <c r="J81" s="22"/>
+      <c r="K81" s="22"/>
+      <c r="L81" s="22"/>
+      <c r="M81" s="22"/>
+    </row>
+    <row r="82" spans="2:13" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B82" s="24" t="s">
         <v>18</v>
       </c>
-      <c r="C77" s="22"/>
-      <c r="D77" s="22"/>
-      <c r="E77" s="22"/>
-      <c r="F77" s="22"/>
-      <c r="G77" s="22"/>
-      <c r="H77" s="22"/>
-      <c r="I77" s="22"/>
-      <c r="J77" s="22"/>
-      <c r="K77" s="12"/>
-      <c r="L77" s="12"/>
-      <c r="M77" s="12"/>
-    </row>
-    <row r="78" spans="1:13" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A78" s="10"/>
-      <c r="B78" s="13" t="s">
+      <c r="C82" s="22"/>
+      <c r="D82" s="22"/>
+      <c r="E82" s="22"/>
+      <c r="F82" s="22"/>
+      <c r="G82" s="22"/>
+      <c r="H82" s="22"/>
+      <c r="I82" s="22"/>
+      <c r="J82" s="22"/>
+      <c r="K82" s="22"/>
+      <c r="L82" s="22"/>
+      <c r="M82" s="22"/>
+    </row>
+    <row r="83" spans="2:13" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B83" s="24" t="s">
+        <v>25</v>
+      </c>
+      <c r="C83" s="22"/>
+      <c r="D83" s="22"/>
+      <c r="E83" s="22"/>
+      <c r="F83" s="22"/>
+      <c r="G83" s="22"/>
+      <c r="H83" s="22"/>
+      <c r="I83" s="22"/>
+      <c r="J83" s="22"/>
+      <c r="K83" s="22"/>
+      <c r="L83" s="22"/>
+      <c r="M83" s="22"/>
+    </row>
+    <row r="84" spans="2:13" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B84" s="24" t="s">
         <v>19</v>
       </c>
-      <c r="C78" s="14"/>
-      <c r="D78" s="14"/>
-      <c r="E78" s="14"/>
-      <c r="F78" s="14"/>
-      <c r="G78" s="14"/>
-      <c r="H78" s="14"/>
-      <c r="I78" s="10"/>
-      <c r="J78" s="10"/>
-      <c r="K78" s="10"/>
-      <c r="L78" s="10"/>
-      <c r="M78" s="10"/>
-    </row>
-    <row r="79" spans="1:13" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A79" s="10"/>
-      <c r="B79" s="14"/>
-      <c r="C79" s="14"/>
-      <c r="D79" s="14"/>
-      <c r="E79" s="14"/>
-      <c r="F79" s="14"/>
-      <c r="G79" s="14"/>
-      <c r="H79" s="14"/>
-      <c r="I79" s="10"/>
-      <c r="J79" s="10"/>
-      <c r="K79" s="10"/>
-      <c r="L79" s="10"/>
-      <c r="M79" s="10"/>
-    </row>
-    <row r="80" spans="1:13" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B80" s="11" t="s">
+      <c r="C84" s="22"/>
+      <c r="D84" s="22"/>
+      <c r="E84" s="22"/>
+      <c r="F84" s="22"/>
+      <c r="G84" s="22"/>
+      <c r="H84" s="22"/>
+      <c r="I84" s="22"/>
+      <c r="J84" s="22"/>
+      <c r="K84" s="22"/>
+      <c r="L84" s="22"/>
+      <c r="M84" s="22"/>
+    </row>
+    <row r="85" spans="2:13" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B85" s="25" t="s">
         <v>20</v>
       </c>
-      <c r="C80" s="15"/>
-      <c r="D80" s="15"/>
-      <c r="E80" s="15"/>
-      <c r="F80" s="16"/>
-      <c r="G80" s="16"/>
-      <c r="H80" s="10"/>
-    </row>
-    <row r="81" spans="2:8" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B81" s="10"/>
-      <c r="C81" s="10"/>
-      <c r="D81" s="10"/>
-      <c r="E81" s="10"/>
-      <c r="F81" s="10"/>
-      <c r="G81" s="10"/>
-      <c r="H81" s="10"/>
-    </row>
-    <row r="82" spans="2:8" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B82" s="11" t="s">
-        <v>21</v>
-      </c>
-      <c r="C82" s="10"/>
-      <c r="D82" s="10"/>
-      <c r="E82" s="10"/>
-      <c r="F82" s="10"/>
-      <c r="G82" s="10"/>
-      <c r="H82" s="10"/>
-    </row>
-    <row r="83" spans="2:8" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B83" s="11" t="s">
-        <v>25</v>
-      </c>
-      <c r="C83" s="10"/>
-      <c r="D83" s="10"/>
-      <c r="E83" s="10"/>
-      <c r="F83" s="10"/>
-      <c r="G83" s="10"/>
-      <c r="H83" s="10"/>
-    </row>
-    <row r="84" spans="2:8" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B84" s="11" t="s">
-        <v>22</v>
-      </c>
-      <c r="C84" s="10"/>
-      <c r="D84" s="10"/>
-      <c r="E84" s="10"/>
-      <c r="F84" s="10"/>
-      <c r="G84" s="10"/>
-      <c r="H84" s="10"/>
-    </row>
-    <row r="85" spans="2:8" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B85" s="17" t="s">
-        <v>23</v>
-      </c>
-      <c r="C85" s="10"/>
-      <c r="D85" s="10"/>
-      <c r="E85" s="10"/>
-      <c r="F85" s="10"/>
-      <c r="G85" s="10"/>
-      <c r="H85" s="10"/>
+      <c r="C85" s="22"/>
+      <c r="D85" s="22"/>
+      <c r="E85" s="22"/>
+      <c r="F85" s="22"/>
+      <c r="G85" s="22"/>
+      <c r="H85" s="22"/>
+      <c r="I85" s="22"/>
+      <c r="J85" s="22"/>
+      <c r="K85" s="22"/>
+      <c r="L85" s="22"/>
+      <c r="M85" s="22"/>
     </row>
   </sheetData>
-  <mergeCells count="10">
+  <mergeCells count="11">
+    <mergeCell ref="B41:B43"/>
+    <mergeCell ref="C41:C43"/>
+    <mergeCell ref="D41:J41"/>
+    <mergeCell ref="D43:J43"/>
+    <mergeCell ref="B75:M75"/>
+    <mergeCell ref="B76:M76"/>
+    <mergeCell ref="B77:M77"/>
     <mergeCell ref="B6:B8"/>
     <mergeCell ref="C6:C8"/>
     <mergeCell ref="D6:J6"/>
     <mergeCell ref="D8:J8"/>
-    <mergeCell ref="B75:J75"/>
-    <mergeCell ref="B77:J77"/>
-    <mergeCell ref="B41:B43"/>
-    <mergeCell ref="C41:C43"/>
-    <mergeCell ref="D41:J41"/>
-    <mergeCell ref="D43:J43"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="B85" r:id="rId1" xr:uid="{E8296B3C-0891-4298-B260-2E9053746E12}"/>
-    <hyperlink ref="B78" r:id="rId2" xr:uid="{C5DE47B4-1D36-4837-95AA-46AE8069022F}"/>
+    <hyperlink ref="B78" r:id="rId1" xr:uid="{E99B2DBB-3654-48CF-894B-543051D83AA2}"/>
+    <hyperlink ref="B85" r:id="rId2" xr:uid="{F4662E07-0D12-46BB-802C-845C04E86A33}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>